<commit_message>
Another update for all English databooks
</commit_message>
<xml_diff>
--- a/inputs/en/LiST countries/AFG_databook.xlsx
+++ b/inputs/en/LiST countries/AFG_databook.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tharindu.wickram\Desktop\LiST Optima bridge\App\en\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9E17A4F1-EB59-4DDC-B975-00C229883EF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{99967EE9-DA48-43A8-8E1C-9658017E9E53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="3670" windowWidth="19200" windowHeight="6530" tabRatio="961" firstSheet="8" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="3670" windowWidth="19200" windowHeight="6530" tabRatio="961" firstSheet="4" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Baseline year population inputs" sheetId="1" r:id="rId1"/>
@@ -9360,7 +9360,7 @@
         <v>11</v>
       </c>
       <c r="C11" s="45">
-        <v>0.17799999999999999</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -9368,7 +9368,7 @@
         <v>12</v>
       </c>
       <c r="C12" s="45">
-        <v>0.61499999999999999</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -11459,19 +11459,19 @@
       </c>
       <c r="D10" s="60">
         <f>IF(ISBLANK(comm_deliv), frac_children_health_facility,1)</f>
-        <v>0.61499999999999999</v>
+        <v>1</v>
       </c>
       <c r="E10" s="60">
         <f>IF(ISBLANK(comm_deliv), frac_children_health_facility,1)</f>
-        <v>0.61499999999999999</v>
+        <v>1</v>
       </c>
       <c r="F10" s="60">
         <f>IF(ISBLANK(comm_deliv), frac_children_health_facility,1)</f>
-        <v>0.61499999999999999</v>
+        <v>1</v>
       </c>
       <c r="G10" s="60">
         <f>IF(ISBLANK(comm_deliv), frac_children_health_facility,1)</f>
-        <v>0.61499999999999999</v>
+        <v>1</v>
       </c>
       <c r="H10" s="61">
         <v>0</v>
@@ -11805,19 +11805,19 @@
       </c>
       <c r="H18" s="60">
         <f>frac_PW_health_facility</f>
-        <v>0.17799999999999999</v>
+        <v>1</v>
       </c>
       <c r="I18" s="60">
         <f>frac_PW_health_facility</f>
-        <v>0.17799999999999999</v>
+        <v>1</v>
       </c>
       <c r="J18" s="60">
         <f>frac_PW_health_facility</f>
-        <v>0.17799999999999999</v>
+        <v>1</v>
       </c>
       <c r="K18" s="60">
         <f>frac_PW_health_facility</f>
-        <v>0.17799999999999999</v>
+        <v>1</v>
       </c>
       <c r="L18" s="61">
         <v>0</v>
@@ -20584,12 +20584,36 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="riIqDHxQDNIc95k8WEEMlpv2yK5yRhEl3GZr9d21PG7QnhNwxgtjaWmZN+9widROwyhXiwQ4XZiTM/cZ2Cl95g==" saltValue="b1Xx0XPjIcbtdUQJGdoNkQ==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="45">
-    <mergeCell ref="B19:B21"/>
-    <mergeCell ref="B2:B4"/>
-    <mergeCell ref="B5:B7"/>
-    <mergeCell ref="B8:B10"/>
-    <mergeCell ref="B11:B13"/>
-    <mergeCell ref="B14:B16"/>
+    <mergeCell ref="B145:B147"/>
+    <mergeCell ref="B148:B150"/>
+    <mergeCell ref="B151:B153"/>
+    <mergeCell ref="B154:B156"/>
+    <mergeCell ref="B128:B130"/>
+    <mergeCell ref="B131:B133"/>
+    <mergeCell ref="B134:B136"/>
+    <mergeCell ref="B137:B139"/>
+    <mergeCell ref="B142:B144"/>
+    <mergeCell ref="B111:B113"/>
+    <mergeCell ref="B114:B116"/>
+    <mergeCell ref="B117:B119"/>
+    <mergeCell ref="B120:B122"/>
+    <mergeCell ref="B125:B127"/>
+    <mergeCell ref="B108:B110"/>
+    <mergeCell ref="B89:B91"/>
+    <mergeCell ref="B92:B94"/>
+    <mergeCell ref="B95:B97"/>
+    <mergeCell ref="B98:B100"/>
+    <mergeCell ref="B101:B103"/>
+    <mergeCell ref="B72:B74"/>
+    <mergeCell ref="B75:B77"/>
+    <mergeCell ref="B78:B80"/>
+    <mergeCell ref="B81:B83"/>
+    <mergeCell ref="B84:B86"/>
+    <mergeCell ref="B55:B57"/>
+    <mergeCell ref="B58:B60"/>
+    <mergeCell ref="B61:B63"/>
+    <mergeCell ref="B64:B66"/>
+    <mergeCell ref="B67:B69"/>
     <mergeCell ref="B42:B44"/>
     <mergeCell ref="B45:B47"/>
     <mergeCell ref="B48:B50"/>
@@ -20599,36 +20623,12 @@
     <mergeCell ref="B31:B33"/>
     <mergeCell ref="B36:B38"/>
     <mergeCell ref="B39:B41"/>
-    <mergeCell ref="B55:B57"/>
-    <mergeCell ref="B58:B60"/>
-    <mergeCell ref="B61:B63"/>
-    <mergeCell ref="B64:B66"/>
-    <mergeCell ref="B67:B69"/>
-    <mergeCell ref="B72:B74"/>
-    <mergeCell ref="B75:B77"/>
-    <mergeCell ref="B78:B80"/>
-    <mergeCell ref="B81:B83"/>
-    <mergeCell ref="B84:B86"/>
-    <mergeCell ref="B108:B110"/>
-    <mergeCell ref="B89:B91"/>
-    <mergeCell ref="B92:B94"/>
-    <mergeCell ref="B95:B97"/>
-    <mergeCell ref="B98:B100"/>
-    <mergeCell ref="B101:B103"/>
-    <mergeCell ref="B111:B113"/>
-    <mergeCell ref="B114:B116"/>
-    <mergeCell ref="B117:B119"/>
-    <mergeCell ref="B120:B122"/>
-    <mergeCell ref="B125:B127"/>
-    <mergeCell ref="B145:B147"/>
-    <mergeCell ref="B148:B150"/>
-    <mergeCell ref="B151:B153"/>
-    <mergeCell ref="B154:B156"/>
-    <mergeCell ref="B128:B130"/>
-    <mergeCell ref="B131:B133"/>
-    <mergeCell ref="B134:B136"/>
-    <mergeCell ref="B137:B139"/>
-    <mergeCell ref="B142:B144"/>
+    <mergeCell ref="B19:B21"/>
+    <mergeCell ref="B2:B4"/>
+    <mergeCell ref="B5:B7"/>
+    <mergeCell ref="B8:B10"/>
+    <mergeCell ref="B11:B13"/>
+    <mergeCell ref="B14:B16"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
@@ -30088,13 +30088,10 @@
         <v>1</v>
       </c>
       <c r="E6" s="90">
-        <f>IF(ISBLANK('Nutritional status distribution'!$E$4),0.64, (0.64*SUM('Nutritional status distribution'!$E$4:$E$5)/(1-0.64*SUM('Nutritional status distribution'!$E$4:$E$5)))
-/ (SUM('Nutritional status distribution'!$E$4:$E$5)/(1-SUM('Nutritional status distribution'!$E$4:$E$5))))</f>
-        <v>0.58868539542060538</v>
+        <v>0.64</v>
       </c>
       <c r="F6" s="90">
-        <f>IF(ISBLANK('Nutritional status distribution'!$F$4),0.64, (0.64*SUM('Nutritional status distribution'!$F$4:$F$5)/(1-0.64*SUM('Nutritional status distribution'!$F$4:$F$5)))/ (SUM('Nutritional status distribution'!$F$4:$F$5)/(1-SUM('Nutritional status distribution'!$F$4:$F$5))))</f>
-        <v>0.53563856384276287</v>
+        <v>0.64</v>
       </c>
       <c r="G6" s="90">
         <v>1</v>
@@ -30111,12 +30108,10 @@
         <v>1</v>
       </c>
       <c r="E7" s="90">
-        <f>IF(ISBLANK('Nutritional status distribution'!$E$4),0.88, (0.88*SUM('Nutritional status distribution'!$E$4:$E$5)/(1-0.88*SUM('Nutritional status distribution'!$E$4:$E$5)))/ (SUM('Nutritional status distribution'!$E$4:$E$5)/(1-SUM('Nutritional status distribution'!$E$4:$E$5))))</f>
-        <v>0.85515264784850797</v>
+        <v>0.88</v>
       </c>
       <c r="F7" s="90">
-        <f>IF(ISBLANK('Nutritional status distribution'!$F$4),0.88, (0.88*SUM('Nutritional status distribution'!$F$4:$F$5)/(1-0.88*SUM('Nutritional status distribution'!$F$4:$F$5)))/ (SUM('Nutritional status distribution'!$F$4:$F$5)/(1-SUM('Nutritional status distribution'!$F$4:$F$5))))</f>
-        <v>0.82633361111851122</v>
+        <v>0.88</v>
       </c>
       <c r="G7" s="90">
         <v>1</v>
@@ -30133,12 +30128,10 @@
         <v>1</v>
       </c>
       <c r="E8" s="90">
-        <f>IF(ISBLANK('Nutritional status distribution'!$E$4),0.88, (0.88*SUM('Nutritional status distribution'!$E$4:$E$5)/(1-0.88*SUM('Nutritional status distribution'!$E$4:$E$5)))/ (SUM('Nutritional status distribution'!$E$4:$E$5)/(1-SUM('Nutritional status distribution'!$E$4:$E$5))))</f>
-        <v>0.85515264784850797</v>
+        <v>0.88</v>
       </c>
       <c r="F8" s="90">
-        <f>IF(ISBLANK('Nutritional status distribution'!$F$4),0.88, (0.88*SUM('Nutritional status distribution'!$F$4:$F$5)/(1-0.88*SUM('Nutritional status distribution'!$F$4:$F$5)))/ (SUM('Nutritional status distribution'!$F$4:$F$5)/(1-SUM('Nutritional status distribution'!$F$4:$F$5))))</f>
-        <v>0.82633361111851122</v>
+        <v>0.88</v>
       </c>
       <c r="G8" s="90">
         <v>1</v>
@@ -30416,12 +30409,10 @@
         <v>1</v>
       </c>
       <c r="E29" s="90">
-        <f>IF(ISBLANK('Nutritional status distribution'!E$4),0.44, (0.44*SUM('Nutritional status distribution'!E$4:E$5)/(1-0.44*SUM('Nutritional status distribution'!E$4:E$5)))/ (SUM('Nutritional status distribution'!E$4:E$5)/(1-SUM('Nutritional status distribution'!E$4:E$5))))</f>
-        <v>0.38746212453399753</v>
+        <v>0.44</v>
       </c>
       <c r="F29" s="90">
-        <f>IF(ISBLANK('Nutritional status distribution'!F$4),0.44, (0.44*SUM('Nutritional status distribution'!F$4:F$5)/(1-0.44*SUM('Nutritional status distribution'!F$4:F$5)))/ (SUM('Nutritional status distribution'!F$4:F$5)/(1-SUM('Nutritional status distribution'!F$4:F$5))))</f>
-        <v>0.3376621809254382</v>
+        <v>0.44</v>
       </c>
       <c r="G29" s="90">
         <f>IF(G6=1,1,G6*0.9)</f>
@@ -30441,12 +30432,10 @@
         <v>1</v>
       </c>
       <c r="E30" s="90">
-        <f>IF(ISBLANK('Nutritional status distribution'!E$4),0.85, (0.85*SUM('Nutritional status distribution'!E$4:E$5)/(1-0.85*SUM('Nutritional status distribution'!E$4:E$5)))/ (SUM('Nutritional status distribution'!E$4:E$5)/(1-SUM('Nutritional status distribution'!E$4:E$5))))</f>
-        <v>0.82020993116114049</v>
+        <v>0.85</v>
       </c>
       <c r="F30" s="90">
-        <f>IF(ISBLANK('Nutritional status distribution'!F$4),0.85, (0.85*SUM('Nutritional status distribution'!F$4:F$5)/(1-0.85*SUM('Nutritional status distribution'!F$4:F$5)))/ (SUM('Nutritional status distribution'!F$4:F$5)/(1-SUM('Nutritional status distribution'!F$4:F$5))))</f>
-        <v>0.78617698802105751</v>
+        <v>0.85</v>
       </c>
       <c r="G30" s="90">
         <f>IF(G7=1,1,G7*0.9)</f>
@@ -30466,12 +30455,10 @@
         <v>1</v>
       </c>
       <c r="E31" s="90">
-        <f>IF(ISBLANK('Nutritional status distribution'!E$4),0.85, (0.85*SUM('Nutritional status distribution'!E$4:E$5)/(1-0.85*SUM('Nutritional status distribution'!E$4:E$5)))/ (SUM('Nutritional status distribution'!E$4:E$5)/(1-SUM('Nutritional status distribution'!E$4:E$5))))</f>
-        <v>0.82020993116114049</v>
+        <v>0.85</v>
       </c>
       <c r="F31" s="90">
-        <f>IF(ISBLANK('Nutritional status distribution'!F$4),0.85, (0.85*SUM('Nutritional status distribution'!F$4:F$5)/(1-0.85*SUM('Nutritional status distribution'!F$4:F$5)))/ (SUM('Nutritional status distribution'!F$4:F$5)/(1-SUM('Nutritional status distribution'!F$4:F$5))))</f>
-        <v>0.78617698802105751</v>
+        <v>0.85</v>
       </c>
       <c r="G31" s="90">
         <f>IF(G8=1,1,G8*0.9)</f>
@@ -30791,12 +30778,10 @@
         <v>1</v>
       </c>
       <c r="E52" s="90">
-        <f>IF(ISBLANK('Nutritional status distribution'!E$4),0.92, (0.92*SUM('Nutritional status distribution'!E$4:E$5)/(1-0.92*SUM('Nutritional status distribution'!E$4:E$5)))/ (SUM('Nutritional status distribution'!E$4:E$5)/(1-SUM('Nutritional status distribution'!E$4:E$5))))</f>
-        <v>0.90251760638280187</v>
+        <v>0.92</v>
       </c>
       <c r="F52" s="90">
-        <f>IF(ISBLANK('Nutritional status distribution'!F$4),0.92, (0.92*SUM('Nutritional status distribution'!F$4:F$5)/(1-0.92*SUM('Nutritional status distribution'!F$4:F$5)))/ (SUM('Nutritional status distribution'!F$4:F$5)/(1-SUM('Nutritional status distribution'!F$4:F$5))))</f>
-        <v>0.88182002386798231</v>
+        <v>0.92</v>
       </c>
       <c r="G52" s="90">
         <f>IF(G6=1,1,G6*1.1)</f>
@@ -30816,12 +30801,10 @@
         <v>1</v>
       </c>
       <c r="E53" s="90">
-        <f>IF(ISBLANK('Nutritional status distribution'!E$4),0.91, (0.91*SUM('Nutritional status distribution'!E$4:E$5)/(1-0.91*SUM('Nutritional status distribution'!E$4:E$5)))/ (SUM('Nutritional status distribution'!E$4:E$5)/(1-SUM('Nutritional status distribution'!E$4:E$5))))</f>
-        <v>0.89059218631972226</v>
+        <v>0.91</v>
       </c>
       <c r="F53" s="90">
-        <f>IF(ISBLANK('Nutritional status distribution'!F$4),0.91, (0.91*SUM('Nutritional status distribution'!F$4:F$5)/(1-0.91*SUM('Nutritional status distribution'!F$4:F$5)))/ (SUM('Nutritional status distribution'!F$4:F$5)/(1-SUM('Nutritional status distribution'!F$4:F$5))))</f>
-        <v>0.86773365807130454</v>
+        <v>0.91</v>
       </c>
       <c r="G53" s="90">
         <f>IF(G7=1,1,G7*1.1)</f>
@@ -30841,12 +30824,10 @@
         <v>1</v>
       </c>
       <c r="E54" s="90">
-        <f>IF(ISBLANK('Nutritional status distribution'!E$4),0.91, (0.91*SUM('Nutritional status distribution'!E$4:E$5)/(1-0.91*SUM('Nutritional status distribution'!E$4:E$5)))/ (SUM('Nutritional status distribution'!E$4:E$5)/(1-SUM('Nutritional status distribution'!E$4:E$5))))</f>
-        <v>0.89059218631972226</v>
+        <v>0.91</v>
       </c>
       <c r="F54" s="90">
-        <f>IF(ISBLANK('Nutritional status distribution'!F$4),0.91, (0.91*SUM('Nutritional status distribution'!F$4:F$5)/(1-0.91*SUM('Nutritional status distribution'!F$4:F$5)))/ (SUM('Nutritional status distribution'!F$4:F$5)/(1-SUM('Nutritional status distribution'!F$4:F$5))))</f>
-        <v>0.86773365807130454</v>
+        <v>0.91</v>
       </c>
       <c r="G54" s="90">
         <f>IF(G8=1,1,G8*1.1)</f>
@@ -40720,177 +40701,4 @@
   <sheetProtection algorithmName="SHA-512" hashValue="tS5A5il384gB8zsJjwidwZIpdVsJo/ah59cRAmnHpig36ZssdSIeiIXxiNqdW+7yhHG743nXUgYflxFLjdX6Kg==" saltValue="H9BMcvjdiLgSEjFGZvTrQw==" spinCount="100000" sheet="1" scenarios="1" selectLockedCells="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100856A3DB4B0A5FF4A85E5854FA9B1BD84" ma:contentTypeVersion="6" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="107b52809c0cc4b5077f1ac81d3c69cc">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5de2aea6-bdc3-4e5f-b0ae-84d85b5764e4" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="82b7e1b740270cfb0676be859a78f3d0" ns2:_="">
-    <xsd:import namespace="5de2aea6-bdc3-4e5f-b0ae-84d85b5764e4"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="5de2aea6-bdc3-4e5f-b0ae-84d85b5764e4" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="10" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="11" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="12" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{28D900F8-F214-4F34-BFC8-2672D57AA098}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{24BC6678-BE46-42A1-A3A5-7425DDF59883}"/>
 </file>
</xml_diff>

<commit_message>
New demo databooks and English versions after new ORs
</commit_message>
<xml_diff>
--- a/inputs/en/LiST countries/AFG_databook.xlsx
+++ b/inputs/en/LiST countries/AFG_databook.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27425"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tharindu.wickram\Desktop\LiST Optima bridge\App\en\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{99967EE9-DA48-43A8-8E1C-9658017E9E53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E725B7C0-E4A8-425F-A152-76F971BF663B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="3670" windowWidth="19200" windowHeight="6530" tabRatio="961" firstSheet="4" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="3670" windowWidth="19200" windowHeight="6530" tabRatio="961" firstSheet="6" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Baseline year population inputs" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="Causes of death" sheetId="3" r:id="rId3"/>
     <sheet name="Nutritional status distribution" sheetId="4" r:id="rId4"/>
     <sheet name="Breastfeeding distribution" sheetId="5" r:id="rId5"/>
-    <sheet name="Time trends" sheetId="6" state="hidden" r:id="rId6"/>
+    <sheet name="Time trends" sheetId="6" r:id="rId6"/>
     <sheet name="Economic loss" sheetId="7" r:id="rId7"/>
     <sheet name="IYCF packages" sheetId="8" r:id="rId8"/>
     <sheet name="Treatment of SAM" sheetId="9" r:id="rId9"/>
@@ -678,8 +678,7 @@
             <rFont val="Arial"/>
           </rPr>
           <t>Tharindu Wickramaarachchi:
-Lassi et al 2020, RR 0.64 (0.44-0.92) 
-RR converted to OR</t>
+OR = 0.89 for stunting [Panjwani et al. 2017 J Nutr</t>
         </r>
       </text>
     </comment>
@@ -692,8 +691,7 @@
             <rFont val="Arial"/>
           </rPr>
           <t>Tharindu Wickramaarachchi:
-Lassi et al 2020, RR 0.64 (0.44-0.92) 
-RR converted to OR</t>
+OR = 0.89 for stunting [Panjwani et al. 2017 J Nutr</t>
         </r>
       </text>
     </comment>
@@ -834,35 +832,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E29" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-1600-00000E000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <color rgb="FF000000"/>
-            <rFont val="Arial"/>
-          </rPr>
-          <t>Tharindu Wickramaarachchi:
-Lassi et al 2020, RR 0.64 (0.44-0.92) 
-RR converted to OR</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="F29" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-1600-00000F000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <color rgb="FF000000"/>
-            <rFont val="Arial"/>
-          </rPr>
-          <t>Tharindu Wickramaarachchi:
-Lassi et al 2020, RR 0.64 (0.44-0.92) 
-RR converted to OR</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B30" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1600-000010000000}">
+    <comment ref="B30" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1600-00000E000000}">
       <text>
         <r>
           <rPr>
@@ -876,7 +846,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E30" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-1600-000011000000}">
+    <comment ref="E30" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-1600-00000F000000}">
       <text>
         <r>
           <rPr>
@@ -890,7 +860,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E31" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-1600-000012000000}">
+    <comment ref="E31" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-1600-000010000000}">
       <text>
         <r>
           <rPr>
@@ -904,7 +874,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A34" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-1600-000013000000}">
+    <comment ref="A34" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-1600-000011000000}">
       <text>
         <r>
           <rPr>
@@ -917,7 +887,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A37" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-1600-000014000000}">
+    <comment ref="A37" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-1600-000012000000}">
       <text>
         <r>
           <rPr>
@@ -930,7 +900,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B44" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-1600-000015000000}">
+    <comment ref="B44" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-1600-000013000000}">
       <text>
         <r>
           <rPr>
@@ -943,7 +913,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A51" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-1600-000016000000}">
+    <comment ref="A51" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-1600-000014000000}">
       <text>
         <r>
           <rPr>
@@ -956,7 +926,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B52" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1600-000017000000}">
+    <comment ref="B52" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1600-000015000000}">
       <text>
         <r>
           <rPr>
@@ -969,35 +939,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E52" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-1600-000018000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <color rgb="FF000000"/>
-            <rFont val="Arial"/>
-          </rPr>
-          <t>Tharindu Wickramaarachchi:
-Lassi et al 2020, RR 0.64 (0.44-0.92) 
-RR converted to OR</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="F52" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-1600-000019000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <color rgb="FF000000"/>
-            <rFont val="Arial"/>
-          </rPr>
-          <t>Tharindu Wickramaarachchi:
-Lassi et al 2020, RR 0.64 (0.44-0.92) 
-RR converted to OR</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B53" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1600-00001A000000}">
+    <comment ref="B53" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1600-000016000000}">
       <text>
         <r>
           <rPr>
@@ -1011,7 +953,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E53" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-1600-00001B000000}">
+    <comment ref="E53" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-1600-000017000000}">
       <text>
         <r>
           <rPr>
@@ -1025,7 +967,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E54" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-1600-00001C000000}">
+    <comment ref="E54" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-1600-000018000000}">
       <text>
         <r>
           <rPr>
@@ -1561,8 +1503,7 @@
             <rFont val="Arial"/>
           </rPr>
           <t>Tharindu Wickramaarachchi:
-RR from the lterature was used.
-RRR = 0.53 (0.40-0.70) for being anaemic [Hutton and Hassan, 2007 Jama [63]]</t>
+Zhao et al 2019, ≥6 months, RR 0.92 (0.87-0.99 )</t>
         </r>
       </text>
     </comment>
@@ -2134,8 +2075,7 @@
             <rFont val="Arial"/>
           </rPr>
           <t>Tharindu Wickramaarachchi:
-Peña‐Rosas et al 2019, anemia RR 0.72 (0.54-0.97)
-If no data for anaemia prev. the use RR otherwise convert RR to OR using prev.</t>
+OR = 0.976 (0.975-0.978) for being anaemic [Barkley et al. 2015, B J Nutrition [80]]</t>
         </r>
       </text>
     </comment>
@@ -2161,8 +2101,7 @@
             <rFont val="Arial"/>
           </rPr>
           <t>Tharindu Wickramaarachchi:
-Larson et al 2021, RR 0.80 (0.70-0.92)
-If no data for anaemia prev. the use RR otherwise convert RR to OR using prev.</t>
+OR = 0.976 (0.975-0.978) for being anaemic [Barkley et al. 2015, B J Nutrition [80]]</t>
         </r>
       </text>
     </comment>
@@ -2188,8 +2127,7 @@
             <rFont val="Arial"/>
           </rPr>
           <t>Tharindu Wickramaarachchi:
-RR from the lterature was used.
-RRR = 0.53 (0.40-0.70) for being anaemic [Hutton and Hassan, 2007 Jama [63]]</t>
+Zhao et al 2019, ≥6 months, RR 0.92 (0.87-0.99 )</t>
         </r>
       </text>
     </comment>
@@ -2652,7 +2590,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C49" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-000052000000}">
+    <comment ref="E42" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-000052000000}">
       <text>
         <r>
           <rPr>
@@ -2661,12 +2599,37 @@
             <rFont val="Arial"/>
           </rPr>
           <t>Tharindu Wickramaarachchi:
-RR from the lterature was used.
-RRR = 0.53 (0.40-0.70) for being anaemic [Hutton and Hassan, 2007 Jama [63]]</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="H50" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-000053000000}">
+OR = 0.976 (0.975-0.978) for being anaemic [Barkley et al. 2015, B J Nutrition [80]]</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E44" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-000053000000}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Arial"/>
+          </rPr>
+          <t>Tharindu Wickramaarachchi:
+OR = 0.976 (0.975-0.978) for being anaemic [Barkley et al. 2015, B J Nutrition [80]]</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C49" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-000054000000}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Arial"/>
+          </rPr>
+          <t>Tharindu Wickramaarachchi:
+Zhao et al 2019, ≥6 months, RR 0.92 (0.87-0.99 )</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="H50" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-000055000000}">
       <text>
         <r>
           <rPr>
@@ -2680,7 +2643,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="I50" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-000054000000}">
+    <comment ref="I50" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-000056000000}">
       <text>
         <r>
           <rPr>
@@ -2694,7 +2657,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J50" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-000055000000}">
+    <comment ref="J50" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-000057000000}">
       <text>
         <r>
           <rPr>
@@ -2708,7 +2671,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="K50" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-000056000000}">
+    <comment ref="K50" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-000058000000}">
       <text>
         <r>
           <rPr>
@@ -2722,7 +2685,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="H51" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-000057000000}">
+    <comment ref="H51" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-000059000000}">
       <text>
         <r>
           <rPr>
@@ -2736,7 +2699,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="I51" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-000058000000}">
+    <comment ref="I51" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-00005A000000}">
       <text>
         <r>
           <rPr>
@@ -2750,7 +2713,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J51" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-000059000000}">
+    <comment ref="J51" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-00005B000000}">
       <text>
         <r>
           <rPr>
@@ -2764,7 +2727,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="K51" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-00005A000000}">
+    <comment ref="K51" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-00005C000000}">
       <text>
         <r>
           <rPr>
@@ -2778,7 +2741,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="H52" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-00005B000000}">
+    <comment ref="H52" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-00005D000000}">
       <text>
         <r>
           <rPr>
@@ -2792,7 +2755,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="I52" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-00005C000000}">
+    <comment ref="I52" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-00005E000000}">
       <text>
         <r>
           <rPr>
@@ -2806,7 +2769,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J52" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-00005D000000}">
+    <comment ref="J52" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-00005F000000}">
       <text>
         <r>
           <rPr>
@@ -2820,7 +2783,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="K52" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-00005E000000}">
+    <comment ref="K52" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-000060000000}">
       <text>
         <r>
           <rPr>
@@ -2834,7 +2797,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="H53" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-00005F000000}">
+    <comment ref="H53" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-000061000000}">
       <text>
         <r>
           <rPr>
@@ -2848,7 +2811,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="I53" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-000060000000}">
+    <comment ref="I53" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-000062000000}">
       <text>
         <r>
           <rPr>
@@ -2862,7 +2825,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J53" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-000061000000}">
+    <comment ref="J53" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-000063000000}">
       <text>
         <r>
           <rPr>
@@ -2876,7 +2839,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="K53" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-000062000000}">
+    <comment ref="K53" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-000064000000}">
       <text>
         <r>
           <rPr>
@@ -2890,7 +2853,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="L54" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-000063000000}">
+    <comment ref="L54" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-000065000000}">
       <text>
         <r>
           <rPr>
@@ -2903,7 +2866,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="M54" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-000064000000}">
+    <comment ref="M54" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-000066000000}">
       <text>
         <r>
           <rPr>
@@ -2916,7 +2879,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="N54" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-000065000000}">
+    <comment ref="N54" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-000067000000}">
       <text>
         <r>
           <rPr>
@@ -2929,7 +2892,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="O54" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-000066000000}">
+    <comment ref="O54" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-000068000000}">
       <text>
         <r>
           <rPr>
@@ -2942,7 +2905,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="L55" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-000067000000}">
+    <comment ref="L55" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-000069000000}">
       <text>
         <r>
           <rPr>
@@ -2955,7 +2918,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="M55" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-000068000000}">
+    <comment ref="M55" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-00006A000000}">
       <text>
         <r>
           <rPr>
@@ -2968,7 +2931,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="N55" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-000069000000}">
+    <comment ref="N55" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-00006B000000}">
       <text>
         <r>
           <rPr>
@@ -2981,7 +2944,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="O55" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-00006A000000}">
+    <comment ref="O55" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-00006C000000}">
       <text>
         <r>
           <rPr>
@@ -2994,7 +2957,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="L56" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-00006B000000}">
+    <comment ref="L56" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-00006D000000}">
       <text>
         <r>
           <rPr>
@@ -3007,7 +2970,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="M56" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-00006C000000}">
+    <comment ref="M56" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-00006E000000}">
       <text>
         <r>
           <rPr>
@@ -3020,7 +2983,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="N56" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-00006D000000}">
+    <comment ref="N56" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-00006F000000}">
       <text>
         <r>
           <rPr>
@@ -3033,7 +2996,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="O56" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-00006E000000}">
+    <comment ref="O56" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-000070000000}">
       <text>
         <r>
           <rPr>
@@ -3046,7 +3009,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C58" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-00006F000000}">
+    <comment ref="C58" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-000071000000}">
       <text>
         <r>
           <rPr>
@@ -3060,7 +3023,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D58" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-000070000000}">
+    <comment ref="D58" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-000072000000}">
       <text>
         <r>
           <rPr>
@@ -3074,7 +3037,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E58" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-000071000000}">
+    <comment ref="E58" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-000073000000}">
       <text>
         <r>
           <rPr>
@@ -3088,7 +3051,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="F58" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-000072000000}">
+    <comment ref="F58" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-000074000000}">
       <text>
         <r>
           <rPr>
@@ -3102,7 +3065,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="G58" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-000073000000}">
+    <comment ref="G58" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-000075000000}">
       <text>
         <r>
           <rPr>
@@ -3116,7 +3079,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="H58" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-000074000000}">
+    <comment ref="H58" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-000076000000}">
       <text>
         <r>
           <rPr>
@@ -3130,7 +3093,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="I58" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-000075000000}">
+    <comment ref="I58" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-000077000000}">
       <text>
         <r>
           <rPr>
@@ -3144,7 +3107,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J58" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-000076000000}">
+    <comment ref="J58" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-000078000000}">
       <text>
         <r>
           <rPr>
@@ -3158,7 +3121,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="K58" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-000077000000}">
+    <comment ref="K58" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-000079000000}">
       <text>
         <r>
           <rPr>
@@ -3172,7 +3135,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="L58" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-000078000000}">
+    <comment ref="L58" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-00007A000000}">
       <text>
         <r>
           <rPr>
@@ -3186,7 +3149,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="M58" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-000079000000}">
+    <comment ref="M58" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-00007B000000}">
       <text>
         <r>
           <rPr>
@@ -3200,7 +3163,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="N58" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-00007A000000}">
+    <comment ref="N58" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-00007C000000}">
       <text>
         <r>
           <rPr>
@@ -3214,7 +3177,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="O58" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-00007B000000}">
+    <comment ref="O58" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-00007D000000}">
       <text>
         <r>
           <rPr>
@@ -3228,7 +3191,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E59" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-00007C000000}">
+    <comment ref="E59" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-00007E000000}">
       <text>
         <r>
           <rPr>
@@ -3241,7 +3204,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="F59" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-00007D000000}">
+    <comment ref="F59" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-00007F000000}">
       <text>
         <r>
           <rPr>
@@ -3254,7 +3217,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="G59" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-00007E000000}">
+    <comment ref="G59" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-000080000000}">
       <text>
         <r>
           <rPr>
@@ -3267,7 +3230,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E61" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-00007F000000}">
+    <comment ref="E61" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-000081000000}">
       <text>
         <r>
           <rPr>
@@ -3280,7 +3243,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="F61" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-000080000000}">
+    <comment ref="F61" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-000082000000}">
       <text>
         <r>
           <rPr>
@@ -3290,6 +3253,32 @@
           </rPr>
           <t xml:space="preserve">Tharindu Wickramaarachchi:
 Wessells et al 2022, iron deficiency anemia), PR 0.36 (0.30-0.44) </t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E65" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-000083000000}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Arial"/>
+          </rPr>
+          <t>Tharindu Wickramaarachchi:
+OR = 0.976 (0.975-0.978) for being anaemic [Barkley et al. 2015, B J Nutrition [80]]</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E67" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1800-000084000000}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Arial"/>
+          </rPr>
+          <t>Tharindu Wickramaarachchi:
+OR = 0.976 (0.975-0.978) for being anaemic [Barkley et al. 2015, B J Nutrition [80]]</t>
         </r>
       </text>
     </comment>
@@ -6929,9 +6918,8 @@
             <color rgb="FF000000"/>
             <rFont val="Arial"/>
           </rPr>
-          <t>Tharindu Wickramaarachchi:
-RR converted to an OR using BF prev.
-Lassi et al 2019, EIBF RR 1.56 (1.37-1.77)</t>
+          <t xml:space="preserve">Tharindu Wickramaarachchi:
+Mahumud et al 2022, EBF OR 1.73 (1.35-2.11) </t>
         </r>
       </text>
     </comment>
@@ -6943,9 +6931,8 @@
             <color rgb="FF000000"/>
             <rFont val="Arial"/>
           </rPr>
-          <t>Tharindu Wickramaarachchi:
-RR converted to an OR using BF prev.
-Lassi et al 2019, EIBF RR 1.56 (1.37-1.77)</t>
+          <t xml:space="preserve">Tharindu Wickramaarachchi:
+Mahumud et al 2022, EBF OR 1.73 (1.35-2.11) </t>
         </r>
       </text>
     </comment>
@@ -6957,9 +6944,8 @@
             <color rgb="FF000000"/>
             <rFont val="Arial"/>
           </rPr>
-          <t>Tharindu Wickramaarachchi:
-RR converted to an OR using BF prev.
-Lassi et al 2019, EIBF RR 1.56 (1.37-1.77)</t>
+          <t xml:space="preserve">Tharindu Wickramaarachchi:
+Mahumud et al 2022, EBF OR 1.73 (1.35-2.11) </t>
         </r>
       </text>
     </comment>
@@ -6971,9 +6957,8 @@
             <color rgb="FF000000"/>
             <rFont val="Arial"/>
           </rPr>
-          <t>Tharindu Wickramaarachchi:
-RR converted to an OR using BF prev.
-Lassi et al 2019, EIBF RR 1.56 (1.37-1.77)</t>
+          <t xml:space="preserve">Tharindu Wickramaarachchi:
+Mahumud et al 2022, EBF OR 1.73 (1.35-2.11) </t>
         </r>
       </text>
     </comment>
@@ -7106,68 +7091,12 @@
             <color rgb="FF000000"/>
             <rFont val="Arial"/>
           </rPr>
-          <t>Tharindu Wickramaarachchi:
-RR converted to an OR using BF prev.
-Lassi et al 2019, EIBF RR 1.56 (1.37-1.77)</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D59" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1300-00000F000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <color rgb="FF000000"/>
-            <rFont val="Arial"/>
-          </rPr>
-          <t>Tharindu Wickramaarachchi:
-RR converted to an OR using BF prev.
-Lassi et al 2019, EIBF RR 1.56 (1.37-1.77)</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="E61" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1300-000010000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <color rgb="FF000000"/>
-            <rFont val="Arial"/>
-          </rPr>
-          <t>Tharindu Wickramaarachchi:
-RR converted to an OR using BF prev.
-Lassi et al 2019, EIBF RR 1.56 (1.37-1.77)</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="E62" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1300-000011000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <color rgb="FF000000"/>
-            <rFont val="Arial"/>
-          </rPr>
-          <t>Tharindu Wickramaarachchi:
-RR converted to an OR using BF prev.
-Lassi et al 2019, EIBF RR 1.56 (1.37-1.77)</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="F64" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1300-000012000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <color rgb="FF000000"/>
-            <rFont val="Arial"/>
-          </rPr>
           <t xml:space="preserve">Tharindu Wickramaarachchi:
 Mahumud et al 2022, EBF OR 1.73 (1.35-2.11) </t>
         </r>
       </text>
     </comment>
-    <comment ref="F65" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1300-000013000000}">
+    <comment ref="D59" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1300-00000F000000}">
       <text>
         <r>
           <rPr>
@@ -7180,7 +7109,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="G67" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1300-000014000000}">
+    <comment ref="E61" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1300-000010000000}">
       <text>
         <r>
           <rPr>
@@ -7193,7 +7122,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="G68" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1300-000015000000}">
+    <comment ref="E62" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1300-000011000000}">
       <text>
         <r>
           <rPr>
@@ -7206,6 +7135,58 @@
         </r>
       </text>
     </comment>
+    <comment ref="F64" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1300-000012000000}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Arial"/>
+          </rPr>
+          <t xml:space="preserve">Tharindu Wickramaarachchi:
+Mahumud et al 2022, EBF OR 1.73 (1.35-2.11) </t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F65" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1300-000013000000}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Arial"/>
+          </rPr>
+          <t xml:space="preserve">Tharindu Wickramaarachchi:
+Mahumud et al 2022, EBF OR 1.73 (1.35-2.11) </t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G67" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1300-000014000000}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Arial"/>
+          </rPr>
+          <t xml:space="preserve">Tharindu Wickramaarachchi:
+Mahumud et al 2022, EBF OR 1.73 (1.35-2.11) </t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G68" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1300-000015000000}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Arial"/>
+          </rPr>
+          <t xml:space="preserve">Tharindu Wickramaarachchi:
+Mahumud et al 2022, EBF OR 1.73 (1.35-2.11) </t>
+        </r>
+      </text>
+    </comment>
     <comment ref="A89" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-1300-000016000000}">
       <text>
         <r>
@@ -7227,9 +7208,8 @@
             <color rgb="FF000000"/>
             <rFont val="Arial"/>
           </rPr>
-          <t>Tharindu Wickramaarachchi:
-RR converted to an OR using BF prev.
-Lassi et al 2019, EIBF RR 1.56 (1.37-1.77)</t>
+          <t xml:space="preserve">Tharindu Wickramaarachchi:
+Mahumud et al 2022, EBF OR 1.73 (1.35-2.11) </t>
         </r>
       </text>
     </comment>
@@ -7241,9 +7221,8 @@
             <color rgb="FF000000"/>
             <rFont val="Arial"/>
           </rPr>
-          <t>Tharindu Wickramaarachchi:
-RR converted to an OR using BF prev.
-Lassi et al 2019, EIBF RR 1.56 (1.37-1.77)</t>
+          <t xml:space="preserve">Tharindu Wickramaarachchi:
+Mahumud et al 2022, EBF OR 1.73 (1.35-2.11) </t>
         </r>
       </text>
     </comment>
@@ -7255,9 +7234,8 @@
             <color rgb="FF000000"/>
             <rFont val="Arial"/>
           </rPr>
-          <t>Tharindu Wickramaarachchi:
-RR converted to an OR using BF prev.
-Lassi et al 2019, EIBF RR 1.56 (1.37-1.77)</t>
+          <t xml:space="preserve">Tharindu Wickramaarachchi:
+Mahumud et al 2022, EBF OR 1.73 (1.35-2.11) </t>
         </r>
       </text>
     </comment>
@@ -7269,9 +7247,8 @@
             <color rgb="FF000000"/>
             <rFont val="Arial"/>
           </rPr>
-          <t>Tharindu Wickramaarachchi:
-RR converted to an OR using BF prev.
-Lassi et al 2019, EIBF RR 1.56 (1.37-1.77)</t>
+          <t xml:space="preserve">Tharindu Wickramaarachchi:
+Mahumud et al 2022, EBF OR 1.73 (1.35-2.11) </t>
         </r>
       </text>
     </comment>
@@ -7358,7 +7335,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2092" uniqueCount="341">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2094" uniqueCount="341">
   <si>
     <t>Baseline year data</t>
   </si>
@@ -9787,7 +9764,7 @@
         <v>166</v>
       </c>
       <c r="B2" s="45">
-        <v>3.3420706456999988E-2</v>
+        <v>0</v>
       </c>
       <c r="C2" s="98">
         <v>0.95</v>
@@ -9810,7 +9787,7 @@
         <v>168</v>
       </c>
       <c r="B3" s="45">
-        <v>0</v>
+        <v>0.14616947995580001</v>
       </c>
       <c r="C3" s="98">
         <v>0.95</v>
@@ -9862,7 +9839,7 @@
         <v>0.95</v>
       </c>
       <c r="D5" s="56">
-        <v>0.18295608825211421</v>
+        <v>0.19409811402666791</v>
       </c>
       <c r="E5" s="56" t="s">
         <v>167</v>
@@ -9971,7 +9948,7 @@
         <v>175</v>
       </c>
       <c r="B10" s="45">
-        <v>0</v>
+        <v>6.7892599999999997E-2</v>
       </c>
       <c r="C10" s="98">
         <v>0.95</v>
@@ -9994,7 +9971,7 @@
         <v>176</v>
       </c>
       <c r="B11" s="98">
-        <v>0</v>
+        <v>6.7892599999999997E-2</v>
       </c>
       <c r="C11" s="98">
         <v>0.95</v>
@@ -10017,7 +9994,7 @@
         <v>177</v>
       </c>
       <c r="B12" s="98">
-        <v>0</v>
+        <v>6.7892599999999997E-2</v>
       </c>
       <c r="C12" s="98">
         <v>0.95</v>
@@ -10040,7 +10017,7 @@
         <v>178</v>
       </c>
       <c r="B13" s="98">
-        <v>0</v>
+        <v>6.7892599999999997E-2</v>
       </c>
       <c r="C13" s="98">
         <v>0.95</v>
@@ -10063,7 +10040,7 @@
         <v>179</v>
       </c>
       <c r="B14" s="45">
-        <v>0</v>
+        <v>6.7892599999999997E-2</v>
       </c>
       <c r="C14" s="98">
         <v>0.95</v>
@@ -10086,7 +10063,7 @@
         <v>180</v>
       </c>
       <c r="B15" s="98">
-        <v>0</v>
+        <v>6.7892599999999997E-2</v>
       </c>
       <c r="C15" s="98">
         <v>0.95</v>
@@ -10109,7 +10086,7 @@
         <v>181</v>
       </c>
       <c r="B16" s="45">
-        <v>0.14616947995580001</v>
+        <v>0.6</v>
       </c>
       <c r="C16" s="98">
         <v>0.95</v>
@@ -10132,7 +10109,7 @@
         <v>182</v>
       </c>
       <c r="B17" s="98">
-        <v>0.6</v>
+        <v>6.5675947999999998E-2</v>
       </c>
       <c r="C17" s="98">
         <v>0.95</v>
@@ -10155,7 +10132,7 @@
         <v>148</v>
       </c>
       <c r="B18" s="98">
-        <v>0</v>
+        <v>6.0830819922510007E-2</v>
       </c>
       <c r="C18" s="98">
         <v>0.95</v>
@@ -10178,7 +10155,7 @@
         <v>151</v>
       </c>
       <c r="B19" s="98">
-        <v>0</v>
+        <v>0.5595194</v>
       </c>
       <c r="C19" s="98">
         <v>0.95</v>
@@ -10224,7 +10201,7 @@
         <v>183</v>
       </c>
       <c r="B21" s="45">
-        <v>0.30872719999999998</v>
+        <v>0.23417370000000001</v>
       </c>
       <c r="C21" s="98">
         <v>0.95</v>
@@ -10270,7 +10247,7 @@
         <v>185</v>
       </c>
       <c r="B23" s="98">
-        <v>8.1247000000000003E-3</v>
+        <v>0</v>
       </c>
       <c r="C23" s="98">
         <v>0.95</v>
@@ -10293,7 +10270,7 @@
         <v>186</v>
       </c>
       <c r="B24" s="45">
-        <v>0.36148058905760999</v>
+        <v>0.46095589698012002</v>
       </c>
       <c r="C24" s="98">
         <v>0.95</v>
@@ -10339,7 +10316,7 @@
         <v>188</v>
       </c>
       <c r="B26" s="45">
-        <v>0</v>
+        <v>6.7892599999999997E-2</v>
       </c>
       <c r="C26" s="98">
         <v>0.95</v>
@@ -10362,7 +10339,7 @@
         <v>189</v>
       </c>
       <c r="B27" s="45">
-        <v>4.2850491051999999E-2</v>
+        <v>0</v>
       </c>
       <c r="C27" s="98">
         <v>0.95</v>
@@ -10385,7 +10362,7 @@
         <v>190</v>
       </c>
       <c r="B28" s="45">
-        <v>0.46226600000000001</v>
+        <v>0.36148058905760999</v>
       </c>
       <c r="C28" s="98">
         <v>0.95</v>
@@ -10454,7 +10431,7 @@
         <v>157</v>
       </c>
       <c r="B31" s="45">
-        <v>9.2499999999999999E-2</v>
+        <v>0.57999999999999996</v>
       </c>
       <c r="C31" s="98">
         <v>0.95</v>
@@ -10477,7 +10454,7 @@
         <v>193</v>
       </c>
       <c r="B32" s="45">
-        <v>0.41937809999999998</v>
+        <v>0</v>
       </c>
       <c r="C32" s="98">
         <v>0.95</v>
@@ -10523,7 +10500,7 @@
         <v>195</v>
       </c>
       <c r="B34" s="45">
-        <v>0.5595194</v>
+        <v>0.57999999999999996</v>
       </c>
       <c r="C34" s="98">
         <v>0.95</v>
@@ -10569,7 +10546,7 @@
         <v>197</v>
       </c>
       <c r="B36" s="45">
-        <v>0</v>
+        <v>0.220586</v>
       </c>
       <c r="C36" s="98">
         <v>0.95</v>
@@ -10592,7 +10569,7 @@
         <v>198</v>
       </c>
       <c r="B37" s="45">
-        <v>0.57999999999999996</v>
+        <v>0</v>
       </c>
       <c r="C37" s="98">
         <v>0.95</v>
@@ -10615,7 +10592,7 @@
         <v>199</v>
       </c>
       <c r="B38" s="45">
-        <v>9.6197400000000002E-2</v>
+        <v>0.46226600000000001</v>
       </c>
       <c r="C38" s="98">
         <v>0.95</v>
@@ -10638,7 +10615,7 @@
         <v>200</v>
       </c>
       <c r="B39" s="45">
-        <v>0.220586</v>
+        <v>0</v>
       </c>
       <c r="C39" s="98">
         <v>0.95</v>
@@ -15990,31 +15967,31 @@
         <v>2024</v>
       </c>
       <c r="B2" s="49">
-        <v>1170332.544</v>
+        <v>1468735</v>
       </c>
       <c r="C2" s="49">
-        <v>2418000</v>
+        <v>2905774.5</v>
       </c>
       <c r="D2" s="49">
-        <v>3820000</v>
+        <v>3950747</v>
       </c>
       <c r="E2" s="49">
-        <v>2482000</v>
+        <v>2532678.5</v>
       </c>
       <c r="F2" s="49">
-        <v>1682000</v>
+        <v>1394378</v>
       </c>
       <c r="G2" s="17">
         <f t="shared" ref="G2:G13" si="0">C2+D2+E2+F2</f>
-        <v>10402000</v>
+        <v>10783578</v>
       </c>
       <c r="H2" s="17">
         <f t="shared" ref="H2:H13" si="1">(B2 + stillbirth*B2/(1000-stillbirth))/(1-abortion)</f>
-        <v>1364977.3702492372</v>
+        <v>1713008.877836532</v>
       </c>
       <c r="I2" s="17">
         <f t="shared" ref="I2:I13" si="2">G2-H2</f>
-        <v>9037022.6297507621</v>
+        <v>9070569.1221634671</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -16023,31 +16000,31 @@
         <v>2025</v>
       </c>
       <c r="B3" s="49">
-        <v>1169993.5759999999</v>
+        <v>1477664</v>
       </c>
       <c r="C3" s="50">
-        <v>2448000</v>
+        <v>2949385</v>
       </c>
       <c r="D3" s="50">
-        <v>3941000</v>
+        <v>4058596.5</v>
       </c>
       <c r="E3" s="50">
-        <v>2579000</v>
+        <v>2659627</v>
       </c>
       <c r="F3" s="50">
-        <v>1750000</v>
+        <v>1437093.5</v>
       </c>
       <c r="G3" s="17">
         <f t="shared" si="0"/>
-        <v>10718000</v>
+        <v>11104702</v>
       </c>
       <c r="H3" s="17">
         <f t="shared" si="1"/>
-        <v>1364582.0265056058</v>
+        <v>1723422.9118659531</v>
       </c>
       <c r="I3" s="17">
         <f t="shared" si="2"/>
-        <v>9353417.9734943938</v>
+        <v>9381279.0881340466</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -16056,31 +16033,31 @@
         <v>2026</v>
       </c>
       <c r="B4" s="49">
-        <v>1172382.3684</v>
+        <v>1493786</v>
       </c>
       <c r="C4" s="50">
-        <v>2462000</v>
+        <v>2998178.5</v>
       </c>
       <c r="D4" s="50">
-        <v>4070000</v>
+        <v>4165697.5</v>
       </c>
       <c r="E4" s="50">
-        <v>2687000</v>
+        <v>2788340.5</v>
       </c>
       <c r="F4" s="50">
-        <v>1816000</v>
+        <v>1483886.5</v>
       </c>
       <c r="G4" s="17">
         <f t="shared" si="0"/>
-        <v>11035000</v>
+        <v>11436103</v>
       </c>
       <c r="H4" s="17">
         <f t="shared" si="1"/>
-        <v>1367368.1128918556</v>
+        <v>1742226.2556471531</v>
       </c>
       <c r="I4" s="17">
         <f t="shared" si="2"/>
-        <v>9667631.8871081434</v>
+        <v>9693876.7443528473</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -16089,31 +16066,31 @@
         <v>2027</v>
       </c>
       <c r="B5" s="49">
-        <v>1173883.0567999999</v>
+        <v>1499799</v>
       </c>
       <c r="C5" s="50">
-        <v>2460000</v>
+        <v>3054535.5</v>
       </c>
       <c r="D5" s="50">
-        <v>4191000</v>
+        <v>4274463.5</v>
       </c>
       <c r="E5" s="50">
-        <v>2804000</v>
+        <v>2917505</v>
       </c>
       <c r="F5" s="50">
-        <v>1880000</v>
+        <v>1536477</v>
       </c>
       <c r="G5" s="17">
         <f t="shared" si="0"/>
-        <v>11335000</v>
+        <v>11782981</v>
       </c>
       <c r="H5" s="17">
         <f t="shared" si="1"/>
-        <v>1369118.3895258745</v>
+        <v>1749239.3127217318</v>
       </c>
       <c r="I5" s="17">
         <f t="shared" si="2"/>
-        <v>9965881.6104741246</v>
+        <v>10033741.687278269</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -16122,31 +16099,31 @@
         <v>2028</v>
       </c>
       <c r="B6" s="49">
-        <v>1174471.0236</v>
+        <v>1505765</v>
       </c>
       <c r="C6" s="50">
-        <v>2452000</v>
+        <v>3129570</v>
       </c>
       <c r="D6" s="50">
-        <v>4301000</v>
+        <v>4368145</v>
       </c>
       <c r="E6" s="50">
-        <v>2926000</v>
+        <v>3046277.5</v>
       </c>
       <c r="F6" s="50">
-        <v>1944000</v>
+        <v>1595305.5</v>
       </c>
       <c r="G6" s="17">
         <f t="shared" si="0"/>
-        <v>11623000</v>
+        <v>12139298</v>
       </c>
       <c r="H6" s="17">
         <f t="shared" si="1"/>
-        <v>1369804.144511133</v>
+        <v>1756197.5529523878</v>
       </c>
       <c r="I6" s="17">
         <f t="shared" si="2"/>
-        <v>10253195.855488867</v>
+        <v>10383100.447047612</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -16155,31 +16132,31 @@
         <v>2029</v>
       </c>
       <c r="B7" s="49">
-        <v>1174149.2531999999</v>
+        <v>1512936</v>
       </c>
       <c r="C7" s="50">
-        <v>2448000</v>
+        <v>3221360</v>
       </c>
       <c r="D7" s="50">
-        <v>4398000</v>
+        <v>4449861</v>
       </c>
       <c r="E7" s="50">
-        <v>3053000</v>
+        <v>3174490.5</v>
       </c>
       <c r="F7" s="50">
-        <v>2011000</v>
+        <v>1660583.5</v>
       </c>
       <c r="G7" s="17">
         <f t="shared" si="0"/>
-        <v>11910000</v>
+        <v>12506295</v>
       </c>
       <c r="H7" s="17">
         <f t="shared" si="1"/>
-        <v>1369428.8586005874</v>
+        <v>1764561.2037559471</v>
       </c>
       <c r="I7" s="17">
         <f t="shared" si="2"/>
-        <v>10540571.141399413</v>
+        <v>10741733.796244053</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -16188,31 +16165,31 @@
         <v>2030</v>
       </c>
       <c r="B8" s="49">
-        <v>1172870.5</v>
+        <v>1521758</v>
       </c>
       <c r="C8" s="50">
-        <v>2455000</v>
+        <v>3310382.5</v>
       </c>
       <c r="D8" s="50">
-        <v>4480000</v>
+        <v>4534810.5</v>
       </c>
       <c r="E8" s="50">
-        <v>3180000</v>
+        <v>3301572</v>
       </c>
       <c r="F8" s="50">
-        <v>2081000</v>
+        <v>1732985</v>
       </c>
       <c r="G8" s="17">
         <f t="shared" si="0"/>
-        <v>12196000</v>
+        <v>12879750</v>
       </c>
       <c r="H8" s="17">
         <f t="shared" si="1"/>
-        <v>1367937.4285031485</v>
+        <v>1774850.4419917583</v>
       </c>
       <c r="I8" s="17">
         <f t="shared" si="2"/>
-        <v>10828062.571496852</v>
+        <v>11104899.558008242</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -16221,31 +16198,31 @@
         <v>2031</v>
       </c>
       <c r="B9" s="49">
-        <v>1173233.0651428569</v>
+        <v>1523392</v>
       </c>
       <c r="C9" s="50">
-        <v>2460285.7142857141</v>
+        <v>3396745</v>
       </c>
       <c r="D9" s="50">
-        <v>4574285.7142857146</v>
+        <v>4618710.5</v>
       </c>
       <c r="E9" s="50">
-        <v>3279714.2857142859</v>
+        <v>3426603</v>
       </c>
       <c r="F9" s="50">
-        <v>2138000</v>
+        <v>1813334.5</v>
       </c>
       <c r="G9" s="17">
         <f t="shared" si="0"/>
-        <v>12452285.714285715</v>
+        <v>13255393</v>
       </c>
       <c r="H9" s="17">
         <f t="shared" si="1"/>
-        <v>1368360.2939679928</v>
+        <v>1776756.2020549315</v>
       </c>
       <c r="I9" s="17">
         <f t="shared" si="2"/>
-        <v>11083925.420317722</v>
+        <v>11478636.797945069</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -16254,31 +16231,31 @@
         <v>2032</v>
       </c>
       <c r="B10" s="49">
-        <v>1173695.8493061219</v>
+        <v>1534556</v>
       </c>
       <c r="C10" s="50">
-        <v>2462040.8163265302</v>
+        <v>3477338</v>
       </c>
       <c r="D10" s="50">
-        <v>4664755.102040817</v>
+        <v>4708517.5</v>
       </c>
       <c r="E10" s="50">
-        <v>3379816.326530613</v>
+        <v>3548918.5</v>
       </c>
       <c r="F10" s="50">
-        <v>2193428.5714285709</v>
+        <v>1902426.5</v>
       </c>
       <c r="G10" s="17">
         <f t="shared" si="0"/>
-        <v>12700040.816326531</v>
+        <v>13637200.5</v>
       </c>
       <c r="H10" s="17">
         <f t="shared" si="1"/>
-        <v>1368900.0464626192</v>
+        <v>1789776.9519602356</v>
       </c>
       <c r="I10" s="17">
         <f t="shared" si="2"/>
-        <v>11331140.769863911</v>
+        <v>11847423.548039764</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -16287,31 +16264,31 @@
         <v>2033</v>
       </c>
       <c r="B11" s="49">
-        <v>1173883.489435568</v>
+        <v>1534932</v>
       </c>
       <c r="C11" s="50">
-        <v>2462046.6472303201</v>
+        <v>3549482.5</v>
       </c>
       <c r="D11" s="50">
-        <v>4749720.1166180763</v>
+        <v>4808255</v>
       </c>
       <c r="E11" s="50">
-        <v>3478790.0874635568</v>
+        <v>3667562.5</v>
       </c>
       <c r="F11" s="50">
-        <v>2247346.9387755101</v>
+        <v>2000292</v>
       </c>
       <c r="G11" s="17">
         <f t="shared" si="0"/>
-        <v>12937903.790087461</v>
+        <v>14025592</v>
       </c>
       <c r="H11" s="17">
         <f t="shared" si="1"/>
-        <v>1369118.8941155854</v>
+        <v>1790215.4867116148</v>
       </c>
       <c r="I11" s="17">
         <f t="shared" si="2"/>
-        <v>11568784.895971876</v>
+        <v>12235376.513288386</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -16320,31 +16297,31 @@
         <v>2034</v>
       </c>
       <c r="B12" s="49">
-        <v>1173883.55124065</v>
+        <v>1540730</v>
       </c>
       <c r="C12" s="50">
-        <v>2462339.0254060798</v>
+        <v>3619308</v>
       </c>
       <c r="D12" s="50">
-        <v>4829537.2761349455</v>
+        <v>4912971.5</v>
       </c>
       <c r="E12" s="50">
-        <v>3575188.6713869232</v>
+        <v>3781202.5</v>
       </c>
       <c r="F12" s="50">
-        <v>2299825.072886297</v>
+        <v>2105961.5</v>
       </c>
       <c r="G12" s="17">
         <f t="shared" si="0"/>
-        <v>13166890.045814246</v>
+        <v>14419443.5</v>
       </c>
       <c r="H12" s="17">
         <f t="shared" si="1"/>
-        <v>1369118.9661998309</v>
+        <v>1796977.785883144</v>
       </c>
       <c r="I12" s="17">
         <f t="shared" si="2"/>
-        <v>11797771.079614416</v>
+        <v>12622465.714116856</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -16353,31 +16330,31 @@
         <v>2035</v>
       </c>
       <c r="B13" s="49">
-        <v>1173799.626617885</v>
+        <v>1544169</v>
       </c>
       <c r="C13" s="50">
-        <v>2463816.0290355198</v>
+        <v>3688461</v>
       </c>
       <c r="D13" s="50">
-        <v>4905042.6012970796</v>
+        <v>5025354.5</v>
       </c>
       <c r="E13" s="50">
-        <v>3667929.9101564828</v>
+        <v>3889516</v>
       </c>
       <c r="F13" s="50">
-        <v>2350657.2261557681</v>
+        <v>2217473.5</v>
       </c>
       <c r="G13" s="17">
         <f t="shared" si="0"/>
-        <v>13387445.76664485</v>
+        <v>14820805</v>
       </c>
       <c r="H13" s="17">
         <f t="shared" si="1"/>
-        <v>1369021.0835839298</v>
+        <v>1800988.7460161019</v>
       </c>
       <c r="I13" s="17">
         <f t="shared" si="2"/>
-        <v>12018424.68306092</v>
+        <v>13019816.253983898</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -16916,7 +16893,7 @@
         <v>145</v>
       </c>
       <c r="D5" s="88">
-        <v>1.56</v>
+        <v>1.73</v>
       </c>
       <c r="E5" s="88">
         <v>1</v>
@@ -16937,7 +16914,7 @@
         <v>146</v>
       </c>
       <c r="D6" s="88">
-        <v>1.56</v>
+        <v>1.73</v>
       </c>
       <c r="E6" s="88">
         <v>1</v>
@@ -16984,7 +16961,7 @@
         <v>1</v>
       </c>
       <c r="E8" s="88">
-        <v>1.56</v>
+        <v>1.73</v>
       </c>
       <c r="F8" s="88">
         <v>1</v>
@@ -17005,7 +16982,7 @@
         <v>1</v>
       </c>
       <c r="E9" s="88">
-        <v>1.56</v>
+        <v>1.73</v>
       </c>
       <c r="F9" s="88">
         <v>1</v>
@@ -18036,7 +18013,7 @@
         <v>145</v>
       </c>
       <c r="D58" s="88">
-        <v>1.37</v>
+        <v>1.35</v>
       </c>
       <c r="E58" s="88">
         <f t="shared" ref="E58:H60" si="1">IF(E5=1,1,E5*0.9)</f>
@@ -18061,7 +18038,7 @@
         <v>146</v>
       </c>
       <c r="D59" s="88">
-        <v>1.37</v>
+        <v>1.35</v>
       </c>
       <c r="E59" s="88">
         <f t="shared" si="1"/>
@@ -18118,7 +18095,7 @@
         <v>1</v>
       </c>
       <c r="E61" s="88">
-        <v>1.37</v>
+        <v>1.35</v>
       </c>
       <c r="F61" s="88">
         <f t="shared" ref="F61:H63" si="3">IF(F8=1,1,F8*0.9)</f>
@@ -18143,7 +18120,7 @@
         <v>1</v>
       </c>
       <c r="E62" s="88">
-        <v>1.37</v>
+        <v>1.35</v>
       </c>
       <c r="F62" s="88">
         <f t="shared" si="3"/>
@@ -19373,7 +19350,7 @@
         <v>145</v>
       </c>
       <c r="D111" s="88">
-        <v>1.77</v>
+        <v>2.11</v>
       </c>
       <c r="E111" s="88">
         <f t="shared" ref="E111:H113" si="11">IF(E5=1,1,E5*1.05)</f>
@@ -19398,7 +19375,7 @@
         <v>146</v>
       </c>
       <c r="D112" s="88">
-        <v>1.77</v>
+        <v>2.11</v>
       </c>
       <c r="E112" s="88">
         <f t="shared" si="11"/>
@@ -19455,7 +19432,7 @@
         <v>1</v>
       </c>
       <c r="E114" s="88">
-        <v>1.77</v>
+        <v>2.11</v>
       </c>
       <c r="F114" s="88">
         <f t="shared" ref="F114:H116" si="13">IF(F8=1,1,F8*1.05)</f>
@@ -19480,7 +19457,7 @@
         <v>1</v>
       </c>
       <c r="E115" s="88">
-        <v>1.77</v>
+        <v>2.11</v>
       </c>
       <c r="F115" s="88">
         <f t="shared" si="13"/>
@@ -20582,7 +20559,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="riIqDHxQDNIc95k8WEEMlpv2yK5yRhEl3GZr9d21PG7QnhNwxgtjaWmZN+9widROwyhXiwQ4XZiTM/cZ2Cl95g==" saltValue="b1Xx0XPjIcbtdUQJGdoNkQ==" spinCount="100000" sheet="1" selectLockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="kNott2FY10++7LpzvuSEUUgvKblMKWlWyTJLQ7V3mUE+D/qQXgkJjdadeNqQ4e0dbATNIZiaZUbYZr3uwCKttQ==" saltValue="MboHEiRAGE0wfo213ZYZVw==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="45">
     <mergeCell ref="B145:B147"/>
     <mergeCell ref="B148:B150"/>
@@ -21844,7 +21821,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="OEa5xq8Dht0iRzVx1fQ1EOJdDm09uSIzQRujIfp/VJ8GNGNECqE8Uut2U6j1omy5Y9ajcKxMUHwzsTWrCb+nAw==" saltValue="Poj67khbkyqhF7WVYd6CsA==" spinCount="100000" sheet="1" selectLockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="a0aX2VfGYRJWLRZcCd5z7lhlUmGJO/EzN4cg0Snhkl/IJQUK1zIL/9W0H+8Dtzn8tPzB4mSWxW65xqA1yiTgOA==" saltValue="o1GVWZzk0+60bY16Wxar5Q==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967292" verticalDpi="4294967292"/>
   <legacyDrawing r:id="rId1"/>
@@ -29979,7 +29956,7 @@
       <c r="I328" s="39"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="rzjjr+eUY+zLxtgvRuigrXBCYk8ZjZeKkvy/Wu7lqFGhk7GKsrVngS9i2Jt2gxX9Fn0pC2b9tyB7+BxRGGivEA==" saltValue="vsQDJsypwJz22iUc18xJ6w==" spinCount="100000" sheet="1" selectLockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="1gEiboypgN1VYdmLYuHEsviiXDH91vsC32xKqzOEbclcsh2pOXs0vX071vry3NRJsC+T2/BNfpXbXWW7dldjVQ==" saltValue="XZihSWmo245BlR0GYalydw==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967292" verticalDpi="4294967292"/>
   <legacyDrawing r:id="rId1"/>
@@ -30088,10 +30065,10 @@
         <v>1</v>
       </c>
       <c r="E6" s="90">
-        <v>0.64</v>
+        <v>0.89</v>
       </c>
       <c r="F6" s="90">
-        <v>0.64</v>
+        <v>0.89</v>
       </c>
       <c r="G6" s="90">
         <v>1</v>
@@ -30409,10 +30386,12 @@
         <v>1</v>
       </c>
       <c r="E29" s="90">
-        <v>0.44</v>
+        <f>E6*0.9</f>
+        <v>0.80100000000000005</v>
       </c>
       <c r="F29" s="90">
-        <v>0.44</v>
+        <f>F6*0.9</f>
+        <v>0.80100000000000005</v>
       </c>
       <c r="G29" s="90">
         <f>IF(G6=1,1,G6*0.9)</f>
@@ -30778,10 +30757,12 @@
         <v>1</v>
       </c>
       <c r="E52" s="90">
-        <v>0.92</v>
+        <f>E6*1.05</f>
+        <v>0.93450000000000011</v>
       </c>
       <c r="F52" s="90">
-        <v>0.92</v>
+        <f>F6*1.05</f>
+        <v>0.93450000000000011</v>
       </c>
       <c r="G52" s="90">
         <f>IF(G6=1,1,G6*1.1)</f>
@@ -31043,7 +31024,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="uxH3qxfpHv3MxEVFpMF959vuuHVMbjUY0YDJlIXIgHOAA25UaRTm/IIjRx7RzEUfWaTP3eP7cZpYIm+m6J8PbA==" saltValue="wm1A0TwV/0DyOIoqtNvfsQ==" spinCount="100000" sheet="1" selectLockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="Z5W0iLQonUXgebQ0oBIAJiknKvZHIMnPuF1vh21+BfR+VnJC7YVzBoFQiTm+hEbHNMOFIRa563Ft7+Jm2vvcKg==" saltValue="MgosxU+mdCbdebb7wBaTKg==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967292" verticalDpi="4294967292"/>
   <legacyDrawing r:id="rId1"/>
@@ -31864,7 +31845,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="lEvf/7Nn9p0s2t120JFgJzNA1BIMAO9h8EmTziKGX5ZA7K3Y+rQ77oXfzNqKwsdbYQwCY96ujjsdxuDmqt1luA==" saltValue="pZcegXbvW/wKpwHEQP8pcw==" spinCount="100000" sheet="1" selectLockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="LnjPs+tiryCjGlxIcCoc9VYZVK7anRAVHCvKud83EfjtgKW0vUQr2FSI3nvdju1neMs4gxoXRQGAXnwHTy0eGQ==" saltValue="uusuOaSrLiI1eiqZNmtU+w==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967292" verticalDpi="4294967292"/>
   <legacyDrawing r:id="rId1"/>
@@ -31939,7 +31920,7 @@
         <v>170</v>
       </c>
       <c r="C3" s="90">
-        <v>0.53</v>
+        <v>0.92</v>
       </c>
       <c r="D3" s="90">
         <v>0.53</v>
@@ -32450,16 +32431,16 @@
         <v>1</v>
       </c>
       <c r="L14" s="90">
-        <v>0.51</v>
+        <v>1</v>
       </c>
       <c r="M14" s="90">
-        <v>0.51</v>
+        <v>1</v>
       </c>
       <c r="N14" s="90">
-        <v>0.51</v>
+        <v>1</v>
       </c>
       <c r="O14" s="90">
-        <v>0.51</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
@@ -32567,48 +32548,37 @@
         <v>1</v>
       </c>
       <c r="E19" s="90">
-        <f t="shared" ref="E19:O19" si="0">0.72</f>
-        <v>0.72</v>
+        <v>0.97599999999999998</v>
       </c>
       <c r="F19" s="90">
-        <f t="shared" si="0"/>
-        <v>0.72</v>
+        <v>0.97599999999999998</v>
       </c>
       <c r="G19" s="90">
-        <f t="shared" si="0"/>
-        <v>0.72</v>
+        <v>0.97599999999999998</v>
       </c>
       <c r="H19" s="90">
-        <f t="shared" si="0"/>
-        <v>0.72</v>
+        <v>0.97599999999999998</v>
       </c>
       <c r="I19" s="90">
-        <f t="shared" si="0"/>
-        <v>0.72</v>
+        <v>0.97599999999999998</v>
       </c>
       <c r="J19" s="90">
-        <f t="shared" si="0"/>
-        <v>0.72</v>
+        <v>0.97599999999999998</v>
       </c>
       <c r="K19" s="90">
-        <f t="shared" si="0"/>
-        <v>0.72</v>
+        <v>0.97599999999999998</v>
       </c>
       <c r="L19" s="90">
-        <f t="shared" si="0"/>
-        <v>0.72</v>
+        <v>0.97599999999999998</v>
       </c>
       <c r="M19" s="90">
-        <f t="shared" si="0"/>
-        <v>0.72</v>
+        <v>0.97599999999999998</v>
       </c>
       <c r="N19" s="90">
-        <f t="shared" si="0"/>
-        <v>0.72</v>
+        <v>0.97599999999999998</v>
       </c>
       <c r="O19" s="90">
-        <f t="shared" si="0"/>
-        <v>0.72</v>
+        <v>0.97599999999999998</v>
       </c>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
@@ -32666,37 +32636,37 @@
         <v>1</v>
       </c>
       <c r="E21" s="90">
-        <v>0.8</v>
+        <v>0.97599999999999998</v>
       </c>
       <c r="F21" s="90">
-        <v>0.8</v>
+        <v>0.97599999999999998</v>
       </c>
       <c r="G21" s="90">
-        <v>0.8</v>
+        <v>0.97599999999999998</v>
       </c>
       <c r="H21" s="90">
-        <v>0.8</v>
+        <v>0.97599999999999998</v>
       </c>
       <c r="I21" s="90">
-        <v>0.8</v>
+        <v>0.97599999999999998</v>
       </c>
       <c r="J21" s="90">
-        <v>0.8</v>
+        <v>0.97599999999999998</v>
       </c>
       <c r="K21" s="90">
-        <v>0.8</v>
+        <v>0.97599999999999998</v>
       </c>
       <c r="L21" s="90">
-        <v>0.8</v>
+        <v>0.97599999999999998</v>
       </c>
       <c r="M21" s="90">
-        <v>0.8</v>
+        <v>0.97599999999999998</v>
       </c>
       <c r="N21" s="90">
-        <v>0.8</v>
+        <v>0.97599999999999998</v>
       </c>
       <c r="O21" s="90">
-        <v>0.8</v>
+        <v>0.97599999999999998</v>
       </c>
     </row>
     <row r="23" spans="1:15" s="92" customFormat="1" ht="13" customHeight="1" x14ac:dyDescent="0.3">
@@ -32757,53 +32727,53 @@
         <v>170</v>
       </c>
       <c r="C26" s="90">
-        <v>0.4</v>
+        <v>0.87</v>
       </c>
       <c r="D26" s="90">
         <v>0.4</v>
       </c>
       <c r="E26" s="90">
-        <f t="shared" ref="E26:O26" si="1">IF(E3=1,1,E3*0.9)</f>
+        <f t="shared" ref="E26:O26" si="0">IF(E3=1,1,E3*0.9)</f>
         <v>1</v>
       </c>
       <c r="F26" s="90">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="G26" s="90">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="H26" s="90">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="I26" s="90">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="J26" s="90">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="K26" s="90">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="L26" s="90">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="M26" s="90">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="N26" s="90">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="O26" s="90">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
     </row>
@@ -32812,23 +32782,23 @@
         <v>175</v>
       </c>
       <c r="C27" s="90">
-        <f t="shared" ref="C27:G33" si="2">IF(C4=1,1,C4*0.9)</f>
+        <f t="shared" ref="C27:G33" si="1">IF(C4=1,1,C4*0.9)</f>
         <v>1</v>
       </c>
       <c r="D27" s="90">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="E27" s="90">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="F27" s="90">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="G27" s="90">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="H27" s="90">
@@ -32844,19 +32814,19 @@
         <v>0.56000000000000005</v>
       </c>
       <c r="L27" s="90">
-        <f t="shared" ref="L27:O30" si="3">IF(L4=1,1,L4*0.9)</f>
+        <f t="shared" ref="L27:O30" si="2">IF(L4=1,1,L4*0.9)</f>
         <v>1</v>
       </c>
       <c r="M27" s="90">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="N27" s="90">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="O27" s="90">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
     </row>
@@ -32865,23 +32835,23 @@
         <v>176</v>
       </c>
       <c r="C28" s="90">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="D28" s="90">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="E28" s="90">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="F28" s="90">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="G28" s="90">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="H28" s="90">
@@ -32897,19 +32867,19 @@
         <v>0.56000000000000005</v>
       </c>
       <c r="L28" s="90">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="M28" s="90">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="N28" s="90">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="O28" s="90">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
     </row>
@@ -32918,23 +32888,23 @@
         <v>177</v>
       </c>
       <c r="C29" s="90">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="D29" s="90">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="E29" s="90">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="F29" s="90">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="G29" s="90">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="H29" s="90">
@@ -32950,19 +32920,19 @@
         <v>0.56000000000000005</v>
       </c>
       <c r="L29" s="90">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="M29" s="90">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="N29" s="90">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="O29" s="90">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
     </row>
@@ -32971,23 +32941,23 @@
         <v>178</v>
       </c>
       <c r="C30" s="90">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="D30" s="90">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="E30" s="90">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="F30" s="90">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="G30" s="90">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="H30" s="90">
@@ -33003,19 +32973,19 @@
         <v>0.56000000000000005</v>
       </c>
       <c r="L30" s="90">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="M30" s="90">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="N30" s="90">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="O30" s="90">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
     </row>
@@ -33024,39 +32994,39 @@
         <v>179</v>
       </c>
       <c r="C31" s="90">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="D31" s="90">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="E31" s="90">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="F31" s="90">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="G31" s="90">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="H31" s="90">
-        <f t="shared" ref="H31:K34" si="4">IF(H8=1,1,H8*0.9)</f>
+        <f t="shared" ref="H31:K34" si="3">IF(H8=1,1,H8*0.9)</f>
         <v>1</v>
       </c>
       <c r="I31" s="90">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="J31" s="90">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="K31" s="90">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="L31" s="90">
@@ -33077,39 +33047,39 @@
         <v>180</v>
       </c>
       <c r="C32" s="90">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="D32" s="90">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="E32" s="90">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="F32" s="90">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="G32" s="90">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="H32" s="90">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="I32" s="90">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="J32" s="90">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="K32" s="90">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="L32" s="90">
@@ -33130,39 +33100,39 @@
         <v>181</v>
       </c>
       <c r="C33" s="90">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="D33" s="90">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="E33" s="90">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="F33" s="90">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="G33" s="90">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="H33" s="90">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="I33" s="90">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="J33" s="90">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="K33" s="90">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="L33" s="90">
@@ -33200,19 +33170,19 @@
         <v>1</v>
       </c>
       <c r="H34" s="90">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="I34" s="90">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="J34" s="90">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="K34" s="90">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="L34" s="90">
@@ -33281,11 +33251,11 @@
         <v>188</v>
       </c>
       <c r="C36" s="90">
-        <f t="shared" ref="C36:D38" si="5">IF(C13=1,1,C13*0.9)</f>
+        <f t="shared" ref="C36:D38" si="4">IF(C13=1,1,C13*0.9)</f>
         <v>1</v>
       </c>
       <c r="D36" s="90">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="E36" s="90">
@@ -33298,35 +33268,35 @@
         <v>0.62</v>
       </c>
       <c r="H36" s="90">
-        <f t="shared" ref="H36:O36" si="6">IF(H13=1,1,H13*0.9)</f>
+        <f t="shared" ref="H36:O36" si="5">IF(H13=1,1,H13*0.9)</f>
         <v>1</v>
       </c>
       <c r="I36" s="90">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="J36" s="90">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="K36" s="90">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="L36" s="90">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="M36" s="90">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="N36" s="90">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="O36" s="90">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
     </row>
@@ -33335,56 +33305,52 @@
         <v>189</v>
       </c>
       <c r="C37" s="90">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="D37" s="90">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="E37" s="90">
-        <f t="shared" ref="E37:K37" si="7">IF(E14=1,1,E14*0.9)</f>
+        <f t="shared" ref="E37:K37" si="6">IF(E14=1,1,E14*0.9)</f>
         <v>1</v>
       </c>
       <c r="F37" s="90">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="G37" s="90">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="H37" s="90">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="I37" s="90">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="J37" s="90">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="K37" s="90">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="L37" s="90">
-        <f>L32</f>
-        <v>0.38</v>
+        <v>1</v>
       </c>
       <c r="M37" s="90">
-        <f>M32</f>
-        <v>0.38</v>
+        <v>1</v>
       </c>
       <c r="N37" s="90">
-        <f>N32</f>
-        <v>0.38</v>
+        <v>1</v>
       </c>
       <c r="O37" s="90">
-        <f>O32</f>
-        <v>0.38</v>
+        <v>1</v>
       </c>
     </row>
     <row r="38" spans="1:15" x14ac:dyDescent="0.25">
@@ -33392,11 +33358,11 @@
         <v>192</v>
       </c>
       <c r="C38" s="90">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="D38" s="90">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="E38" s="90">
@@ -33406,39 +33372,39 @@
         <v>0.3</v>
       </c>
       <c r="G38" s="90">
-        <f t="shared" ref="G38:O38" si="8">IF(G15=1,1,G15*0.9)</f>
+        <f t="shared" ref="G38:O38" si="7">IF(G15=1,1,G15*0.9)</f>
         <v>1</v>
       </c>
       <c r="H38" s="90">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="I38" s="90">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="J38" s="90">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="K38" s="90">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="L38" s="90">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="M38" s="90">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="N38" s="90">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="O38" s="90">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
     </row>
@@ -33453,55 +33419,55 @@
         <v>172</v>
       </c>
       <c r="C41" s="90">
-        <f t="shared" ref="C41:O41" si="9">IF(C18=1,1,C18*0.9)</f>
+        <f t="shared" ref="C41:O41" si="8">IF(C18=1,1,C18*0.9)</f>
         <v>1</v>
       </c>
       <c r="D41" s="90">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="E41" s="90">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="F41" s="90">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="G41" s="90">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="H41" s="90">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="I41" s="90">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="J41" s="90">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="K41" s="90">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="L41" s="90">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="M41" s="90">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="N41" s="90">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="O41" s="90">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
     </row>
@@ -33510,45 +33476,45 @@
         <v>173</v>
       </c>
       <c r="C42" s="90">
-        <f t="shared" ref="C42:D44" si="10">IF(C19=1,1,C19*0.9)</f>
+        <f t="shared" ref="C42:D44" si="9">IF(C19=1,1,C19*0.9)</f>
         <v>1</v>
       </c>
       <c r="D42" s="90">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v>1</v>
       </c>
       <c r="E42" s="90">
-        <v>0.54</v>
+        <v>0.97499999999999998</v>
       </c>
       <c r="F42" s="90">
-        <v>0.54</v>
+        <v>0.97499999999999998</v>
       </c>
       <c r="G42" s="90">
-        <v>0.54</v>
+        <v>0.97499999999999998</v>
       </c>
       <c r="H42" s="90">
-        <v>0.54</v>
+        <v>0.97499999999999998</v>
       </c>
       <c r="I42" s="90">
-        <v>0.54</v>
+        <v>0.97499999999999998</v>
       </c>
       <c r="J42" s="90">
-        <v>0.54</v>
+        <v>0.97499999999999998</v>
       </c>
       <c r="K42" s="90">
-        <v>0.54</v>
+        <v>0.97499999999999998</v>
       </c>
       <c r="L42" s="90">
-        <v>0.54</v>
+        <v>0.97499999999999998</v>
       </c>
       <c r="M42" s="90">
-        <v>0.54</v>
+        <v>0.97499999999999998</v>
       </c>
       <c r="N42" s="90">
-        <v>0.54</v>
+        <v>0.97499999999999998</v>
       </c>
       <c r="O42" s="90">
-        <v>0.54</v>
+        <v>0.97499999999999998</v>
       </c>
     </row>
     <row r="43" spans="1:15" x14ac:dyDescent="0.25">
@@ -33556,55 +33522,55 @@
         <v>174</v>
       </c>
       <c r="C43" s="90">
+        <f t="shared" si="9"/>
+        <v>1</v>
+      </c>
+      <c r="D43" s="90">
+        <f t="shared" si="9"/>
+        <v>1</v>
+      </c>
+      <c r="E43" s="90">
+        <f t="shared" ref="E43:O43" si="10">IF(E20=1,1,E20*0.9)</f>
+        <v>1</v>
+      </c>
+      <c r="F43" s="90">
         <f t="shared" si="10"/>
         <v>1</v>
       </c>
-      <c r="D43" s="90">
+      <c r="G43" s="90">
         <f t="shared" si="10"/>
         <v>1</v>
       </c>
-      <c r="E43" s="90">
-        <f t="shared" ref="E43:O43" si="11">IF(E20=1,1,E20*0.9)</f>
-        <v>1</v>
-      </c>
-      <c r="F43" s="90">
-        <f t="shared" si="11"/>
-        <v>1</v>
-      </c>
-      <c r="G43" s="90">
-        <f t="shared" si="11"/>
-        <v>1</v>
-      </c>
       <c r="H43" s="90">
-        <f t="shared" si="11"/>
+        <f t="shared" si="10"/>
         <v>1</v>
       </c>
       <c r="I43" s="90">
-        <f t="shared" si="11"/>
+        <f t="shared" si="10"/>
         <v>1</v>
       </c>
       <c r="J43" s="90">
-        <f t="shared" si="11"/>
+        <f t="shared" si="10"/>
         <v>1</v>
       </c>
       <c r="K43" s="90">
-        <f t="shared" si="11"/>
+        <f t="shared" si="10"/>
         <v>1</v>
       </c>
       <c r="L43" s="90">
-        <f t="shared" si="11"/>
+        <f t="shared" si="10"/>
         <v>1</v>
       </c>
       <c r="M43" s="90">
-        <f t="shared" si="11"/>
+        <f t="shared" si="10"/>
         <v>1</v>
       </c>
       <c r="N43" s="90">
-        <f t="shared" si="11"/>
+        <f t="shared" si="10"/>
         <v>1</v>
       </c>
       <c r="O43" s="90">
-        <f t="shared" si="11"/>
+        <f t="shared" si="10"/>
         <v>1</v>
       </c>
     </row>
@@ -33613,45 +33579,45 @@
         <v>182</v>
       </c>
       <c r="C44" s="90">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v>1</v>
       </c>
       <c r="D44" s="90">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v>1</v>
       </c>
       <c r="E44" s="90">
-        <v>0.7</v>
+        <v>0.97499999999999998</v>
       </c>
       <c r="F44" s="90">
-        <v>0.7</v>
+        <v>0.97499999999999998</v>
       </c>
       <c r="G44" s="90">
-        <v>0.7</v>
+        <v>0.97499999999999998</v>
       </c>
       <c r="H44" s="90">
-        <v>0.7</v>
+        <v>0.97499999999999998</v>
       </c>
       <c r="I44" s="90">
-        <v>0.7</v>
+        <v>0.97499999999999998</v>
       </c>
       <c r="J44" s="90">
-        <v>0.7</v>
+        <v>0.97499999999999998</v>
       </c>
       <c r="K44" s="90">
-        <v>0.7</v>
+        <v>0.97499999999999998</v>
       </c>
       <c r="L44" s="90">
-        <v>0.7</v>
+        <v>0.97499999999999998</v>
       </c>
       <c r="M44" s="90">
-        <v>0.7</v>
+        <v>0.97499999999999998</v>
       </c>
       <c r="N44" s="90">
-        <v>0.7</v>
+        <v>0.97499999999999998</v>
       </c>
       <c r="O44" s="90">
-        <v>0.7</v>
+        <v>0.97499999999999998</v>
       </c>
     </row>
     <row r="46" spans="1:15" s="92" customFormat="1" ht="13" customHeight="1" x14ac:dyDescent="0.3">
@@ -33712,53 +33678,53 @@
         <v>170</v>
       </c>
       <c r="C49" s="90">
-        <v>0.7</v>
+        <v>0.99</v>
       </c>
       <c r="D49" s="90">
         <v>0.7</v>
       </c>
       <c r="E49" s="90">
-        <f t="shared" ref="E49:O49" si="12">IF(E3=1,1,E3*1.05)</f>
+        <f t="shared" ref="E49:O49" si="11">IF(E3=1,1,E3*1.05)</f>
         <v>1</v>
       </c>
       <c r="F49" s="90">
-        <f t="shared" si="12"/>
+        <f t="shared" si="11"/>
         <v>1</v>
       </c>
       <c r="G49" s="90">
-        <f t="shared" si="12"/>
+        <f t="shared" si="11"/>
         <v>1</v>
       </c>
       <c r="H49" s="90">
-        <f t="shared" si="12"/>
+        <f t="shared" si="11"/>
         <v>1</v>
       </c>
       <c r="I49" s="90">
-        <f t="shared" si="12"/>
+        <f t="shared" si="11"/>
         <v>1</v>
       </c>
       <c r="J49" s="90">
-        <f t="shared" si="12"/>
+        <f t="shared" si="11"/>
         <v>1</v>
       </c>
       <c r="K49" s="90">
-        <f t="shared" si="12"/>
+        <f t="shared" si="11"/>
         <v>1</v>
       </c>
       <c r="L49" s="90">
-        <f t="shared" si="12"/>
+        <f t="shared" si="11"/>
         <v>1</v>
       </c>
       <c r="M49" s="90">
-        <f t="shared" si="12"/>
+        <f t="shared" si="11"/>
         <v>1</v>
       </c>
       <c r="N49" s="90">
-        <f t="shared" si="12"/>
+        <f t="shared" si="11"/>
         <v>1</v>
       </c>
       <c r="O49" s="90">
-        <f t="shared" si="12"/>
+        <f t="shared" si="11"/>
         <v>1</v>
       </c>
     </row>
@@ -33767,23 +33733,23 @@
         <v>175</v>
       </c>
       <c r="C50" s="90">
-        <f t="shared" ref="C50:G56" si="13">IF(C4=1,1,C4*1.05)</f>
+        <f t="shared" ref="C50:G56" si="12">IF(C4=1,1,C4*1.05)</f>
         <v>1</v>
       </c>
       <c r="D50" s="90">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>1</v>
       </c>
       <c r="E50" s="90">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>1</v>
       </c>
       <c r="F50" s="90">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>1</v>
       </c>
       <c r="G50" s="90">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>1</v>
       </c>
       <c r="H50" s="90">
@@ -33799,19 +33765,19 @@
         <v>0.95</v>
       </c>
       <c r="L50" s="90">
-        <f t="shared" ref="L50:O53" si="14">IF(L4=1,1,L4*1.05)</f>
+        <f t="shared" ref="L50:O53" si="13">IF(L4=1,1,L4*1.05)</f>
         <v>1</v>
       </c>
       <c r="M50" s="90">
-        <f t="shared" si="14"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="N50" s="90">
-        <f t="shared" si="14"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="O50" s="90">
-        <f t="shared" si="14"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
     </row>
@@ -33820,23 +33786,23 @@
         <v>176</v>
       </c>
       <c r="C51" s="90">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>1</v>
       </c>
       <c r="D51" s="90">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>1</v>
       </c>
       <c r="E51" s="90">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>1</v>
       </c>
       <c r="F51" s="90">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>1</v>
       </c>
       <c r="G51" s="90">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>1</v>
       </c>
       <c r="H51" s="90">
@@ -33852,19 +33818,19 @@
         <v>0.95</v>
       </c>
       <c r="L51" s="90">
-        <f t="shared" si="14"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="M51" s="90">
-        <f t="shared" si="14"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="N51" s="90">
-        <f t="shared" si="14"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="O51" s="90">
-        <f t="shared" si="14"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
     </row>
@@ -33873,23 +33839,23 @@
         <v>177</v>
       </c>
       <c r="C52" s="90">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>1</v>
       </c>
       <c r="D52" s="90">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>1</v>
       </c>
       <c r="E52" s="90">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>1</v>
       </c>
       <c r="F52" s="90">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>1</v>
       </c>
       <c r="G52" s="90">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>1</v>
       </c>
       <c r="H52" s="90">
@@ -33905,19 +33871,19 @@
         <v>0.95</v>
       </c>
       <c r="L52" s="90">
-        <f t="shared" si="14"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="M52" s="90">
-        <f t="shared" si="14"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="N52" s="90">
-        <f t="shared" si="14"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="O52" s="90">
-        <f t="shared" si="14"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
     </row>
@@ -33926,23 +33892,23 @@
         <v>178</v>
       </c>
       <c r="C53" s="90">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>1</v>
       </c>
       <c r="D53" s="90">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>1</v>
       </c>
       <c r="E53" s="90">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>1</v>
       </c>
       <c r="F53" s="90">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>1</v>
       </c>
       <c r="G53" s="90">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>1</v>
       </c>
       <c r="H53" s="90">
@@ -33958,19 +33924,19 @@
         <v>0.95</v>
       </c>
       <c r="L53" s="90">
-        <f t="shared" si="14"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="M53" s="90">
-        <f t="shared" si="14"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="N53" s="90">
-        <f t="shared" si="14"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="O53" s="90">
-        <f t="shared" si="14"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
     </row>
@@ -33979,39 +33945,39 @@
         <v>179</v>
       </c>
       <c r="C54" s="90">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>1</v>
       </c>
       <c r="D54" s="90">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>1</v>
       </c>
       <c r="E54" s="90">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>1</v>
       </c>
       <c r="F54" s="90">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>1</v>
       </c>
       <c r="G54" s="90">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>1</v>
       </c>
       <c r="H54" s="90">
-        <f t="shared" ref="H54:K57" si="15">IF(H8=1,1,H8*1.05)</f>
+        <f t="shared" ref="H54:K57" si="14">IF(H8=1,1,H8*1.05)</f>
         <v>1</v>
       </c>
       <c r="I54" s="90">
-        <f t="shared" si="15"/>
+        <f t="shared" si="14"/>
         <v>1</v>
       </c>
       <c r="J54" s="90">
-        <f t="shared" si="15"/>
+        <f t="shared" si="14"/>
         <v>1</v>
       </c>
       <c r="K54" s="90">
-        <f t="shared" si="15"/>
+        <f t="shared" si="14"/>
         <v>1</v>
       </c>
       <c r="L54" s="90">
@@ -34032,39 +33998,39 @@
         <v>180</v>
       </c>
       <c r="C55" s="90">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>1</v>
       </c>
       <c r="D55" s="90">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>1</v>
       </c>
       <c r="E55" s="90">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>1</v>
       </c>
       <c r="F55" s="90">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>1</v>
       </c>
       <c r="G55" s="90">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>1</v>
       </c>
       <c r="H55" s="90">
-        <f t="shared" si="15"/>
+        <f t="shared" si="14"/>
         <v>1</v>
       </c>
       <c r="I55" s="90">
-        <f t="shared" si="15"/>
+        <f t="shared" si="14"/>
         <v>1</v>
       </c>
       <c r="J55" s="90">
-        <f t="shared" si="15"/>
+        <f t="shared" si="14"/>
         <v>1</v>
       </c>
       <c r="K55" s="90">
-        <f t="shared" si="15"/>
+        <f t="shared" si="14"/>
         <v>1</v>
       </c>
       <c r="L55" s="90">
@@ -34085,39 +34051,39 @@
         <v>181</v>
       </c>
       <c r="C56" s="90">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>1</v>
       </c>
       <c r="D56" s="90">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>1</v>
       </c>
       <c r="E56" s="90">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>1</v>
       </c>
       <c r="F56" s="90">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>1</v>
       </c>
       <c r="G56" s="90">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>1</v>
       </c>
       <c r="H56" s="90">
-        <f t="shared" si="15"/>
+        <f t="shared" si="14"/>
         <v>1</v>
       </c>
       <c r="I56" s="90">
-        <f t="shared" si="15"/>
+        <f t="shared" si="14"/>
         <v>1</v>
       </c>
       <c r="J56" s="90">
-        <f t="shared" si="15"/>
+        <f t="shared" si="14"/>
         <v>1</v>
       </c>
       <c r="K56" s="90">
-        <f t="shared" si="15"/>
+        <f t="shared" si="14"/>
         <v>1</v>
       </c>
       <c r="L56" s="90">
@@ -34156,19 +34122,19 @@
         <v>1</v>
       </c>
       <c r="H57" s="90">
-        <f t="shared" si="15"/>
+        <f t="shared" si="14"/>
         <v>1</v>
       </c>
       <c r="I57" s="90">
-        <f t="shared" si="15"/>
+        <f t="shared" si="14"/>
         <v>1</v>
       </c>
       <c r="J57" s="90">
-        <f t="shared" si="15"/>
+        <f t="shared" si="14"/>
         <v>1</v>
       </c>
       <c r="K57" s="90">
-        <f t="shared" si="15"/>
+        <f t="shared" si="14"/>
         <v>1</v>
       </c>
       <c r="L57" s="90">
@@ -34237,11 +34203,11 @@
         <v>188</v>
       </c>
       <c r="C59" s="90">
-        <f t="shared" ref="C59:D61" si="16">IF(C13=1,1,C13*1.05)</f>
+        <f t="shared" ref="C59:D61" si="15">IF(C13=1,1,C13*1.05)</f>
         <v>1</v>
       </c>
       <c r="D59" s="90">
-        <f t="shared" si="16"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="E59" s="90">
@@ -34254,35 +34220,35 @@
         <v>0.77</v>
       </c>
       <c r="H59" s="90">
-        <f t="shared" ref="H59:O59" si="17">IF(H13=1,1,H13*1.05)</f>
+        <f t="shared" ref="H59:O59" si="16">IF(H13=1,1,H13*1.05)</f>
         <v>1</v>
       </c>
       <c r="I59" s="90">
-        <f t="shared" si="17"/>
+        <f t="shared" si="16"/>
         <v>1</v>
       </c>
       <c r="J59" s="90">
-        <f t="shared" si="17"/>
+        <f t="shared" si="16"/>
         <v>1</v>
       </c>
       <c r="K59" s="90">
-        <f t="shared" si="17"/>
+        <f t="shared" si="16"/>
         <v>1</v>
       </c>
       <c r="L59" s="90">
-        <f t="shared" si="17"/>
+        <f t="shared" si="16"/>
         <v>1</v>
       </c>
       <c r="M59" s="90">
-        <f t="shared" si="17"/>
+        <f t="shared" si="16"/>
         <v>1</v>
       </c>
       <c r="N59" s="90">
-        <f t="shared" si="17"/>
+        <f t="shared" si="16"/>
         <v>1</v>
       </c>
       <c r="O59" s="90">
-        <f t="shared" si="17"/>
+        <f t="shared" si="16"/>
         <v>1</v>
       </c>
     </row>
@@ -34291,56 +34257,52 @@
         <v>189</v>
       </c>
       <c r="C60" s="90">
-        <f t="shared" si="16"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="D60" s="90">
-        <f t="shared" si="16"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="E60" s="90">
-        <f t="shared" ref="E60:K60" si="18">IF(E14=1,1,E14*1.05)</f>
+        <f t="shared" ref="E60:K60" si="17">IF(E14=1,1,E14*1.05)</f>
         <v>1</v>
       </c>
       <c r="F60" s="90">
-        <f t="shared" si="18"/>
+        <f t="shared" si="17"/>
         <v>1</v>
       </c>
       <c r="G60" s="90">
-        <f t="shared" si="18"/>
+        <f t="shared" si="17"/>
         <v>1</v>
       </c>
       <c r="H60" s="90">
-        <f t="shared" si="18"/>
+        <f t="shared" si="17"/>
         <v>1</v>
       </c>
       <c r="I60" s="90">
-        <f t="shared" si="18"/>
+        <f t="shared" si="17"/>
         <v>1</v>
       </c>
       <c r="J60" s="90">
-        <f t="shared" si="18"/>
+        <f t="shared" si="17"/>
         <v>1</v>
       </c>
       <c r="K60" s="90">
-        <f t="shared" si="18"/>
+        <f t="shared" si="17"/>
         <v>1</v>
       </c>
       <c r="L60" s="90">
-        <f>L54</f>
-        <v>0.7</v>
+        <v>1</v>
       </c>
       <c r="M60" s="90">
-        <f>M54</f>
-        <v>0.7</v>
+        <v>1</v>
       </c>
       <c r="N60" s="90">
-        <f>N54</f>
-        <v>0.7</v>
+        <v>1</v>
       </c>
       <c r="O60" s="90">
-        <f>O54</f>
-        <v>0.7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="61" spans="1:15" x14ac:dyDescent="0.25">
@@ -34348,11 +34310,11 @@
         <v>192</v>
       </c>
       <c r="C61" s="90">
-        <f t="shared" si="16"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="D61" s="90">
-        <f t="shared" si="16"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="E61" s="90">
@@ -34362,39 +34324,39 @@
         <v>0.44</v>
       </c>
       <c r="G61" s="90">
-        <f t="shared" ref="G61:O61" si="19">IF(G15=1,1,G15*1.05)</f>
+        <f t="shared" ref="G61:O61" si="18">IF(G15=1,1,G15*1.05)</f>
         <v>1</v>
       </c>
       <c r="H61" s="90">
-        <f t="shared" si="19"/>
+        <f t="shared" si="18"/>
         <v>1</v>
       </c>
       <c r="I61" s="90">
-        <f t="shared" si="19"/>
+        <f t="shared" si="18"/>
         <v>1</v>
       </c>
       <c r="J61" s="90">
-        <f t="shared" si="19"/>
+        <f t="shared" si="18"/>
         <v>1</v>
       </c>
       <c r="K61" s="90">
-        <f t="shared" si="19"/>
+        <f t="shared" si="18"/>
         <v>1</v>
       </c>
       <c r="L61" s="90">
-        <f t="shared" si="19"/>
+        <f t="shared" si="18"/>
         <v>1</v>
       </c>
       <c r="M61" s="90">
-        <f t="shared" si="19"/>
+        <f t="shared" si="18"/>
         <v>1</v>
       </c>
       <c r="N61" s="90">
-        <f t="shared" si="19"/>
+        <f t="shared" si="18"/>
         <v>1</v>
       </c>
       <c r="O61" s="90">
-        <f t="shared" si="19"/>
+        <f t="shared" si="18"/>
         <v>1</v>
       </c>
     </row>
@@ -34409,55 +34371,55 @@
         <v>172</v>
       </c>
       <c r="C64" s="90">
-        <f t="shared" ref="C64:O64" si="20">IF(C18=1,1,C18*1.05)</f>
+        <f t="shared" ref="C64:O64" si="19">IF(C18=1,1,C18*1.05)</f>
         <v>1</v>
       </c>
       <c r="D64" s="90">
-        <f t="shared" si="20"/>
+        <f t="shared" si="19"/>
         <v>1</v>
       </c>
       <c r="E64" s="90">
-        <f t="shared" si="20"/>
+        <f t="shared" si="19"/>
         <v>1</v>
       </c>
       <c r="F64" s="90">
-        <f t="shared" si="20"/>
+        <f t="shared" si="19"/>
         <v>1</v>
       </c>
       <c r="G64" s="90">
-        <f t="shared" si="20"/>
+        <f t="shared" si="19"/>
         <v>1</v>
       </c>
       <c r="H64" s="90">
-        <f t="shared" si="20"/>
+        <f t="shared" si="19"/>
         <v>1</v>
       </c>
       <c r="I64" s="90">
-        <f t="shared" si="20"/>
+        <f t="shared" si="19"/>
         <v>1</v>
       </c>
       <c r="J64" s="90">
-        <f t="shared" si="20"/>
+        <f t="shared" si="19"/>
         <v>1</v>
       </c>
       <c r="K64" s="90">
-        <f t="shared" si="20"/>
+        <f t="shared" si="19"/>
         <v>1</v>
       </c>
       <c r="L64" s="90">
-        <f t="shared" si="20"/>
+        <f t="shared" si="19"/>
         <v>1</v>
       </c>
       <c r="M64" s="90">
-        <f t="shared" si="20"/>
+        <f t="shared" si="19"/>
         <v>1</v>
       </c>
       <c r="N64" s="90">
-        <f t="shared" si="20"/>
+        <f t="shared" si="19"/>
         <v>1</v>
       </c>
       <c r="O64" s="90">
-        <f t="shared" si="20"/>
+        <f t="shared" si="19"/>
         <v>1</v>
       </c>
     </row>
@@ -34466,45 +34428,45 @@
         <v>173</v>
       </c>
       <c r="C65" s="90">
-        <f t="shared" ref="C65:D67" si="21">IF(C19=1,1,C19*1.05)</f>
+        <f t="shared" ref="C65:D67" si="20">IF(C19=1,1,C19*1.05)</f>
         <v>1</v>
       </c>
       <c r="D65" s="90">
-        <f t="shared" si="21"/>
+        <f t="shared" si="20"/>
         <v>1</v>
       </c>
       <c r="E65" s="90">
-        <v>0.97</v>
+        <v>0.97799999999999998</v>
       </c>
       <c r="F65" s="90">
-        <v>0.97</v>
+        <v>0.97799999999999998</v>
       </c>
       <c r="G65" s="90">
-        <v>0.97</v>
+        <v>0.97799999999999998</v>
       </c>
       <c r="H65" s="90">
-        <v>0.97</v>
+        <v>0.97799999999999998</v>
       </c>
       <c r="I65" s="90">
-        <v>0.97</v>
+        <v>0.97799999999999998</v>
       </c>
       <c r="J65" s="90">
-        <v>0.97</v>
+        <v>0.97799999999999998</v>
       </c>
       <c r="K65" s="90">
-        <v>0.97</v>
+        <v>0.97799999999999998</v>
       </c>
       <c r="L65" s="90">
-        <v>0.97</v>
+        <v>0.97799999999999998</v>
       </c>
       <c r="M65" s="90">
-        <v>0.97</v>
+        <v>0.97799999999999998</v>
       </c>
       <c r="N65" s="90">
-        <v>0.97</v>
+        <v>0.97799999999999998</v>
       </c>
       <c r="O65" s="90">
-        <v>0.97</v>
+        <v>0.97799999999999998</v>
       </c>
     </row>
     <row r="66" spans="2:15" x14ac:dyDescent="0.25">
@@ -34512,55 +34474,55 @@
         <v>174</v>
       </c>
       <c r="C66" s="90">
+        <f t="shared" si="20"/>
+        <v>1</v>
+      </c>
+      <c r="D66" s="90">
+        <f t="shared" si="20"/>
+        <v>1</v>
+      </c>
+      <c r="E66" s="90">
+        <f t="shared" ref="E66:O66" si="21">IF(E20=1,1,E20*1.05)</f>
+        <v>1</v>
+      </c>
+      <c r="F66" s="90">
         <f t="shared" si="21"/>
         <v>1</v>
       </c>
-      <c r="D66" s="90">
+      <c r="G66" s="90">
         <f t="shared" si="21"/>
         <v>1</v>
       </c>
-      <c r="E66" s="90">
-        <f t="shared" ref="E66:O66" si="22">IF(E20=1,1,E20*1.05)</f>
-        <v>1</v>
-      </c>
-      <c r="F66" s="90">
-        <f t="shared" si="22"/>
-        <v>1</v>
-      </c>
-      <c r="G66" s="90">
-        <f t="shared" si="22"/>
-        <v>1</v>
-      </c>
       <c r="H66" s="90">
-        <f t="shared" si="22"/>
+        <f t="shared" si="21"/>
         <v>1</v>
       </c>
       <c r="I66" s="90">
-        <f t="shared" si="22"/>
+        <f t="shared" si="21"/>
         <v>1</v>
       </c>
       <c r="J66" s="90">
-        <f t="shared" si="22"/>
+        <f t="shared" si="21"/>
         <v>1</v>
       </c>
       <c r="K66" s="90">
-        <f t="shared" si="22"/>
+        <f t="shared" si="21"/>
         <v>1</v>
       </c>
       <c r="L66" s="90">
-        <f t="shared" si="22"/>
+        <f t="shared" si="21"/>
         <v>1</v>
       </c>
       <c r="M66" s="90">
-        <f t="shared" si="22"/>
+        <f t="shared" si="21"/>
         <v>1</v>
       </c>
       <c r="N66" s="90">
-        <f t="shared" si="22"/>
+        <f t="shared" si="21"/>
         <v>1</v>
       </c>
       <c r="O66" s="90">
-        <f t="shared" si="22"/>
+        <f t="shared" si="21"/>
         <v>1</v>
       </c>
     </row>
@@ -34569,51 +34531,49 @@
         <v>182</v>
       </c>
       <c r="C67" s="90">
-        <f t="shared" si="21"/>
+        <f t="shared" si="20"/>
         <v>1</v>
       </c>
       <c r="D67" s="90">
-        <f t="shared" si="21"/>
+        <f t="shared" si="20"/>
         <v>1</v>
       </c>
       <c r="E67" s="90">
-        <v>0.92</v>
+        <v>0.97799999999999998</v>
       </c>
       <c r="F67" s="90">
-        <v>0.92</v>
+        <v>0.97799999999999998</v>
       </c>
       <c r="G67" s="90">
-        <v>0.92</v>
+        <v>0.97799999999999998</v>
       </c>
       <c r="H67" s="90">
-        <v>0.92</v>
+        <v>0.97799999999999998</v>
       </c>
       <c r="I67" s="90">
-        <v>0.92</v>
+        <v>0.97799999999999998</v>
       </c>
       <c r="J67" s="90">
-        <v>0.92</v>
+        <v>0.97799999999999998</v>
       </c>
       <c r="K67" s="90">
-        <v>0.92</v>
+        <v>0.97799999999999998</v>
       </c>
       <c r="L67" s="90">
-        <v>0.92</v>
+        <v>0.97799999999999998</v>
       </c>
       <c r="M67" s="90">
-        <v>0.92</v>
+        <v>0.97799999999999998</v>
       </c>
       <c r="N67" s="90">
-        <v>0.92</v>
+        <v>0.97799999999999998</v>
       </c>
       <c r="O67" s="90">
-        <f>IF(ISBLANK('Nutritional status distribution'!O$14),0.92,(0.92*'Nutritional status distribution'!O$14/(1-0.92*'Nutritional status distribution'!O$14))
-/ ('Nutritional status distribution'!O$14/(1-'Nutritional status distribution'!O$14)))</f>
-        <v>0.86883525708289611</v>
+        <v>0.97799999999999998</v>
       </c>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="QTNrTNcX0LQnvnw9OcFIuF8iiKsb7nBsadUCrO1kCxqB4CvEkER3v8YCwNBmR8txM/1IAuOQ/zC/vA8HLWjOhA==" saltValue="f5+QlQPEjGE24L/HhPaCMQ==" spinCount="100000" sheet="1" selectLockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="Z+I5w7Zv8b/t9kdTHtfTBlYoSm79UCEUpz3ShmnqEGsFIWvoyqli8qZ/O3UtxFRtNUOisgC6wk7M7CD5q+6g2w==" saltValue="qncMJDCOHin5ZX0oUaABDg==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967292" verticalDpi="4294967292"/>
   <legacyDrawing r:id="rId1"/>
@@ -34895,7 +34855,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="ZIjv20oIFeX8hEAP3JXu7+FjYQdIWvRgXIH4IkxRsMm14MAW5JMg2x9QOPJ7rc+IAMFEDvKO0XCydnz4Atw3VA==" saltValue="eIHIWivrA2mRyU/FI0KAAQ==" spinCount="100000" sheet="1" selectLockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="TSrwgMfue31l5YKH5YC63gNl/EJnr5ZJbUkDIAIpA9VCbqMkKC4yV7Qlzd02MRVNDQ406JZzgd4mO0azU8HKbQ==" saltValue="P3gP/2fV5vANzIL7NniDMg==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <legacyDrawing r:id="rId1"/>
@@ -38623,7 +38583,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="gIF3gzcRwMevsVP9JM+eFJliWIfkjL6RYnVy29HH1zFwKTB/eJc1NVFGROY84dwrfqcI+B8KpOZ1waT1qDgCXQ==" saltValue="0Itsi1W8Rg+oXl6coWpocw==" spinCount="100000" sheet="1" selectLockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="ogxQtq/9g6OeNkiNBs6ghJq8+LdVqsoK1CbSDtbSeFSK0ebg4cqAnXfIn86tuaNowgHjhLbE7woQSAqVYa5K1w==" saltValue="QFHNUEWTAfsZg09RvHfUXA==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967292" verticalDpi="4294967292"/>
   <legacyDrawing r:id="rId1"/>
@@ -39127,7 +39087,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="SSCu+FR+SN+siPEoAiap+3g3Z0SGqFtJklZqGSbEJvGKfBY2J7BHBpfevFvAYPx8Hf15tBeGKZdJ4ehQEpyLRg==" saltValue="A0PmMaoo+OfazXy7x4UxVw==" spinCount="100000" sheet="1" selectLockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="bFi4UO/MYSy1ocOot5y7JdpTLSj3VYrhdtuVEmlekdzp7NtFBQZX4yNIi9A9S9nFic+mLseFiB4QMgSz7PmPmQ==" saltValue="0Yi1KsKDfpD+pl5y1FWoHw==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
 </worksheet>
@@ -40467,7 +40427,9 @@
         <v>78</v>
       </c>
       <c r="C5" s="47"/>
-      <c r="D5" s="47"/>
+      <c r="D5" s="47" t="s">
+        <v>149</v>
+      </c>
       <c r="E5" s="38" t="str">
         <f>IF(E$7="","",E$7)</f>
         <v/>
@@ -40478,7 +40440,9 @@
         <v>79</v>
       </c>
       <c r="C6" s="47"/>
-      <c r="D6" s="47"/>
+      <c r="D6" s="47" t="s">
+        <v>149</v>
+      </c>
       <c r="E6" s="38" t="str">
         <f>IF(E$7="","",E$7)</f>
         <v/>
@@ -40701,4 +40665,177 @@
   <sheetProtection algorithmName="SHA-512" hashValue="tS5A5il384gB8zsJjwidwZIpdVsJo/ah59cRAmnHpig36ZssdSIeiIXxiNqdW+7yhHG743nXUgYflxFLjdX6Kg==" saltValue="H9BMcvjdiLgSEjFGZvTrQw==" spinCount="100000" sheet="1" scenarios="1" selectLockedCells="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100856A3DB4B0A5FF4A85E5854FA9B1BD84" ma:contentTypeVersion="6" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="107b52809c0cc4b5077f1ac81d3c69cc">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5de2aea6-bdc3-4e5f-b0ae-84d85b5764e4" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="82b7e1b740270cfb0676be859a78f3d0" ns2:_="">
+    <xsd:import namespace="5de2aea6-bdc3-4e5f-b0ae-84d85b5764e4"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="5de2aea6-bdc3-4e5f-b0ae-84d85b5764e4" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="10" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="11" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="12" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BD5E8882-0615-453B-8A7B-3E777EC54E25}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6640C4EA-3EE7-491A-98B6-71B785ABC1DC}"/>
 </file>
</xml_diff>

<commit_message>
databooks updated for MMS and IFA fortification for wheat
</commit_message>
<xml_diff>
--- a/inputs/en/LiST countries/AFG_databook.xlsx
+++ b/inputs/en/LiST countries/AFG_databook.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tharindu.wickram\Desktop\LiST Optima bridge\App\en\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E725B7C0-E4A8-425F-A152-76F971BF663B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B593B8A0-CA87-4ED1-AB6F-14F8980B7798}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="3670" windowWidth="19200" windowHeight="6530" tabRatio="961" firstSheet="6" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="3670" windowWidth="19200" windowHeight="6530" tabRatio="961" firstSheet="6" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Baseline year population inputs" sheetId="1" r:id="rId1"/>
@@ -91,7 +91,7 @@
     <definedName name="term_SGA">'Baseline year population inputs'!$C$47</definedName>
     <definedName name="U5_mortality">'Baseline year population inputs'!$C$39</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" concurrentCalc="0"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -2088,7 +2088,8 @@
             <rFont val="Arial"/>
           </rPr>
           <t>Tharindu Wickramaarachchi:
-Insufficient published research on the intervention’s effect on the outcome.</t>
+Insufficient published research on the intervention’s effect on the outcome.
+Thereofre, set effect of rice = effect of wheat</t>
         </r>
       </text>
     </comment>
@@ -7335,7 +7336,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2094" uniqueCount="341">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2102" uniqueCount="341">
   <si>
     <t>Baseline year data</t>
   </si>
@@ -9379,7 +9380,7 @@
         <v>16</v>
       </c>
       <c r="C17" s="45">
-        <v>0.7</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -9387,7 +9388,7 @@
         <v>17</v>
       </c>
       <c r="C18" s="45">
-        <v>0.05</v>
+        <v>0.98</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -9395,7 +9396,7 @@
         <v>18</v>
       </c>
       <c r="C19" s="45">
-        <v>0.05</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -9404,7 +9405,7 @@
       </c>
       <c r="C20" s="46">
         <f>1-frac_rice-frac_wheat-frac_maize</f>
-        <v>0.20000000000000007</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -10634,7 +10635,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="7vflRb+A4U2pEdxn7m/v0lFZNI78qfZXbnYBjV1V9XLM+tHWxQCvL8xYVSz8kIygwB6Bp0chVfPhUDXzL0eOkw==" saltValue="BwzbjGZ5GxwK0BvfdhnvSQ==" spinCount="100000" sheet="1" selectLockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="SwqShMKjZ/Tc3FrdHQz/MjdsWftRTk85s02s32k0tDk98bBhXaGhkqbuII/OivPUJtqXOhQ4ck/oX/RBAeMIgQ==" saltValue="RORLzDUZEp7fquGh4DZ5hw==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967292" verticalDpi="4294967292"/>
   <legacyDrawing r:id="rId1"/>
@@ -10704,23 +10705,39 @@
       <c r="C5" s="47"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="57"/>
-      <c r="B6" s="58"/>
+      <c r="A6" s="57" t="s">
+        <v>191</v>
+      </c>
+      <c r="B6" s="58" t="s">
+        <v>192</v>
+      </c>
       <c r="C6" s="58"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="57"/>
-      <c r="B7" s="58"/>
+      <c r="A7" s="57" t="s">
+        <v>188</v>
+      </c>
+      <c r="B7" s="58" t="s">
+        <v>192</v>
+      </c>
       <c r="C7" s="58"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="57"/>
-      <c r="B8" s="58"/>
+      <c r="A8" s="57" t="s">
+        <v>200</v>
+      </c>
+      <c r="B8" s="58" t="s">
+        <v>192</v>
+      </c>
       <c r="C8" s="58"/>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="57"/>
-      <c r="B9" s="58"/>
+      <c r="A9" s="57" t="s">
+        <v>193</v>
+      </c>
+      <c r="B9" s="58" t="s">
+        <v>192</v>
+      </c>
       <c r="C9" s="58"/>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -12261,47 +12278,47 @@
       </c>
       <c r="E30" s="60">
         <f t="shared" ref="E30:O30" si="0">frac_maize</f>
-        <v>0.05</v>
+        <v>0.01</v>
       </c>
       <c r="F30" s="60">
         <f t="shared" si="0"/>
-        <v>0.05</v>
+        <v>0.01</v>
       </c>
       <c r="G30" s="60">
         <f t="shared" si="0"/>
-        <v>0.05</v>
+        <v>0.01</v>
       </c>
       <c r="H30" s="60">
         <f t="shared" si="0"/>
-        <v>0.05</v>
+        <v>0.01</v>
       </c>
       <c r="I30" s="60">
         <f t="shared" si="0"/>
-        <v>0.05</v>
+        <v>0.01</v>
       </c>
       <c r="J30" s="60">
         <f t="shared" si="0"/>
-        <v>0.05</v>
+        <v>0.01</v>
       </c>
       <c r="K30" s="60">
         <f t="shared" si="0"/>
-        <v>0.05</v>
+        <v>0.01</v>
       </c>
       <c r="L30" s="60">
         <f t="shared" si="0"/>
-        <v>0.05</v>
+        <v>0.01</v>
       </c>
       <c r="M30" s="60">
         <f t="shared" si="0"/>
-        <v>0.05</v>
+        <v>0.01</v>
       </c>
       <c r="N30" s="60">
         <f t="shared" si="0"/>
-        <v>0.05</v>
+        <v>0.01</v>
       </c>
       <c r="O30" s="60">
         <f t="shared" si="0"/>
-        <v>0.05</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="31" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -12316,47 +12333,47 @@
       </c>
       <c r="E31" s="60">
         <f t="shared" ref="E31:O31" si="1">frac_rice</f>
-        <v>0.7</v>
+        <v>0.01</v>
       </c>
       <c r="F31" s="60">
         <f t="shared" si="1"/>
-        <v>0.7</v>
+        <v>0.01</v>
       </c>
       <c r="G31" s="60">
         <f t="shared" si="1"/>
-        <v>0.7</v>
+        <v>0.01</v>
       </c>
       <c r="H31" s="60">
         <f t="shared" si="1"/>
-        <v>0.7</v>
+        <v>0.01</v>
       </c>
       <c r="I31" s="60">
         <f t="shared" si="1"/>
-        <v>0.7</v>
+        <v>0.01</v>
       </c>
       <c r="J31" s="60">
         <f t="shared" si="1"/>
-        <v>0.7</v>
+        <v>0.01</v>
       </c>
       <c r="K31" s="60">
         <f t="shared" si="1"/>
-        <v>0.7</v>
+        <v>0.01</v>
       </c>
       <c r="L31" s="60">
         <f t="shared" si="1"/>
-        <v>0.7</v>
+        <v>0.01</v>
       </c>
       <c r="M31" s="60">
         <f t="shared" si="1"/>
-        <v>0.7</v>
+        <v>0.01</v>
       </c>
       <c r="N31" s="60">
         <f t="shared" si="1"/>
-        <v>0.7</v>
+        <v>0.01</v>
       </c>
       <c r="O31" s="60">
         <f t="shared" si="1"/>
-        <v>0.7</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="32" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -12371,47 +12388,47 @@
       </c>
       <c r="E32" s="60">
         <f t="shared" ref="E32:O32" si="2">frac_wheat</f>
-        <v>0.05</v>
+        <v>0.98</v>
       </c>
       <c r="F32" s="60">
         <f t="shared" si="2"/>
-        <v>0.05</v>
+        <v>0.98</v>
       </c>
       <c r="G32" s="60">
         <f t="shared" si="2"/>
-        <v>0.05</v>
+        <v>0.98</v>
       </c>
       <c r="H32" s="60">
         <f t="shared" si="2"/>
-        <v>0.05</v>
+        <v>0.98</v>
       </c>
       <c r="I32" s="60">
         <f t="shared" si="2"/>
-        <v>0.05</v>
+        <v>0.98</v>
       </c>
       <c r="J32" s="60">
         <f t="shared" si="2"/>
-        <v>0.05</v>
+        <v>0.98</v>
       </c>
       <c r="K32" s="60">
         <f t="shared" si="2"/>
-        <v>0.05</v>
+        <v>0.98</v>
       </c>
       <c r="L32" s="60">
         <f t="shared" si="2"/>
-        <v>0.05</v>
+        <v>0.98</v>
       </c>
       <c r="M32" s="60">
         <f t="shared" si="2"/>
-        <v>0.05</v>
+        <v>0.98</v>
       </c>
       <c r="N32" s="60">
         <f t="shared" si="2"/>
-        <v>0.05</v>
+        <v>0.98</v>
       </c>
       <c r="O32" s="60">
         <f t="shared" si="2"/>
-        <v>0.05</v>
+        <v>0.98</v>
       </c>
     </row>
     <row r="33" spans="2:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -20561,6 +20578,42 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="kNott2FY10++7LpzvuSEUUgvKblMKWlWyTJLQ7V3mUE+D/qQXgkJjdadeNqQ4e0dbATNIZiaZUbYZr3uwCKttQ==" saltValue="MboHEiRAGE0wfo213ZYZVw==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="45">
+    <mergeCell ref="B19:B21"/>
+    <mergeCell ref="B2:B4"/>
+    <mergeCell ref="B5:B7"/>
+    <mergeCell ref="B8:B10"/>
+    <mergeCell ref="B11:B13"/>
+    <mergeCell ref="B14:B16"/>
+    <mergeCell ref="B42:B44"/>
+    <mergeCell ref="B45:B47"/>
+    <mergeCell ref="B48:B50"/>
+    <mergeCell ref="B22:B24"/>
+    <mergeCell ref="B25:B27"/>
+    <mergeCell ref="B28:B30"/>
+    <mergeCell ref="B31:B33"/>
+    <mergeCell ref="B36:B38"/>
+    <mergeCell ref="B39:B41"/>
+    <mergeCell ref="B55:B57"/>
+    <mergeCell ref="B58:B60"/>
+    <mergeCell ref="B61:B63"/>
+    <mergeCell ref="B64:B66"/>
+    <mergeCell ref="B67:B69"/>
+    <mergeCell ref="B72:B74"/>
+    <mergeCell ref="B75:B77"/>
+    <mergeCell ref="B78:B80"/>
+    <mergeCell ref="B81:B83"/>
+    <mergeCell ref="B84:B86"/>
+    <mergeCell ref="B108:B110"/>
+    <mergeCell ref="B89:B91"/>
+    <mergeCell ref="B92:B94"/>
+    <mergeCell ref="B95:B97"/>
+    <mergeCell ref="B98:B100"/>
+    <mergeCell ref="B101:B103"/>
+    <mergeCell ref="B111:B113"/>
+    <mergeCell ref="B114:B116"/>
+    <mergeCell ref="B117:B119"/>
+    <mergeCell ref="B120:B122"/>
+    <mergeCell ref="B125:B127"/>
     <mergeCell ref="B145:B147"/>
     <mergeCell ref="B148:B150"/>
     <mergeCell ref="B151:B153"/>
@@ -20570,42 +20623,6 @@
     <mergeCell ref="B134:B136"/>
     <mergeCell ref="B137:B139"/>
     <mergeCell ref="B142:B144"/>
-    <mergeCell ref="B111:B113"/>
-    <mergeCell ref="B114:B116"/>
-    <mergeCell ref="B117:B119"/>
-    <mergeCell ref="B120:B122"/>
-    <mergeCell ref="B125:B127"/>
-    <mergeCell ref="B108:B110"/>
-    <mergeCell ref="B89:B91"/>
-    <mergeCell ref="B92:B94"/>
-    <mergeCell ref="B95:B97"/>
-    <mergeCell ref="B98:B100"/>
-    <mergeCell ref="B101:B103"/>
-    <mergeCell ref="B72:B74"/>
-    <mergeCell ref="B75:B77"/>
-    <mergeCell ref="B78:B80"/>
-    <mergeCell ref="B81:B83"/>
-    <mergeCell ref="B84:B86"/>
-    <mergeCell ref="B55:B57"/>
-    <mergeCell ref="B58:B60"/>
-    <mergeCell ref="B61:B63"/>
-    <mergeCell ref="B64:B66"/>
-    <mergeCell ref="B67:B69"/>
-    <mergeCell ref="B42:B44"/>
-    <mergeCell ref="B45:B47"/>
-    <mergeCell ref="B48:B50"/>
-    <mergeCell ref="B22:B24"/>
-    <mergeCell ref="B25:B27"/>
-    <mergeCell ref="B28:B30"/>
-    <mergeCell ref="B31:B33"/>
-    <mergeCell ref="B36:B38"/>
-    <mergeCell ref="B39:B41"/>
-    <mergeCell ref="B19:B21"/>
-    <mergeCell ref="B2:B4"/>
-    <mergeCell ref="B5:B7"/>
-    <mergeCell ref="B8:B10"/>
-    <mergeCell ref="B11:B13"/>
-    <mergeCell ref="B14:B16"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
@@ -32431,16 +32448,20 @@
         <v>1</v>
       </c>
       <c r="L14" s="90">
-        <v>1</v>
+        <f>L8</f>
+        <v>0.51</v>
       </c>
       <c r="M14" s="90">
-        <v>1</v>
+        <f>M8</f>
+        <v>0.51</v>
       </c>
       <c r="N14" s="90">
-        <v>1</v>
+        <f>N8</f>
+        <v>0.51</v>
       </c>
       <c r="O14" s="90">
-        <v>1</v>
+        <f>O8</f>
+        <v>0.51</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
@@ -32592,37 +32613,48 @@
         <v>1</v>
       </c>
       <c r="E20" s="90">
-        <v>1</v>
+        <f t="shared" ref="E20:O20" si="0">E19</f>
+        <v>0.97599999999999998</v>
       </c>
       <c r="F20" s="90">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0.97599999999999998</v>
       </c>
       <c r="G20" s="90">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0.97599999999999998</v>
       </c>
       <c r="H20" s="90">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0.97599999999999998</v>
       </c>
       <c r="I20" s="90">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0.97599999999999998</v>
       </c>
       <c r="J20" s="90">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0.97599999999999998</v>
       </c>
       <c r="K20" s="90">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0.97599999999999998</v>
       </c>
       <c r="L20" s="90">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0.97599999999999998</v>
       </c>
       <c r="M20" s="90">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0.97599999999999998</v>
       </c>
       <c r="N20" s="90">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0.97599999999999998</v>
       </c>
       <c r="O20" s="90">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0.97599999999999998</v>
       </c>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
@@ -32733,47 +32765,47 @@
         <v>0.4</v>
       </c>
       <c r="E26" s="90">
-        <f t="shared" ref="E26:O26" si="0">IF(E3=1,1,E3*0.9)</f>
+        <f t="shared" ref="E26:O26" si="1">IF(E3=1,1,E3*0.9)</f>
         <v>1</v>
       </c>
       <c r="F26" s="90">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="G26" s="90">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="H26" s="90">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="I26" s="90">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="J26" s="90">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="K26" s="90">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="L26" s="90">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="M26" s="90">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="N26" s="90">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="O26" s="90">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
     </row>
@@ -32782,23 +32814,23 @@
         <v>175</v>
       </c>
       <c r="C27" s="90">
-        <f t="shared" ref="C27:G33" si="1">IF(C4=1,1,C4*0.9)</f>
+        <f t="shared" ref="C27:G33" si="2">IF(C4=1,1,C4*0.9)</f>
         <v>1</v>
       </c>
       <c r="D27" s="90">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="E27" s="90">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="F27" s="90">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="G27" s="90">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="H27" s="90">
@@ -32814,19 +32846,19 @@
         <v>0.56000000000000005</v>
       </c>
       <c r="L27" s="90">
-        <f t="shared" ref="L27:O30" si="2">IF(L4=1,1,L4*0.9)</f>
+        <f t="shared" ref="L27:O30" si="3">IF(L4=1,1,L4*0.9)</f>
         <v>1</v>
       </c>
       <c r="M27" s="90">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="N27" s="90">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="O27" s="90">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
     </row>
@@ -32835,23 +32867,23 @@
         <v>176</v>
       </c>
       <c r="C28" s="90">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="D28" s="90">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="E28" s="90">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="F28" s="90">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="G28" s="90">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="H28" s="90">
@@ -32867,19 +32899,19 @@
         <v>0.56000000000000005</v>
       </c>
       <c r="L28" s="90">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="M28" s="90">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="N28" s="90">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="O28" s="90">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
     </row>
@@ -32888,23 +32920,23 @@
         <v>177</v>
       </c>
       <c r="C29" s="90">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="D29" s="90">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="E29" s="90">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="F29" s="90">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="G29" s="90">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="H29" s="90">
@@ -32920,19 +32952,19 @@
         <v>0.56000000000000005</v>
       </c>
       <c r="L29" s="90">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="M29" s="90">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="N29" s="90">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="O29" s="90">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
     </row>
@@ -32941,23 +32973,23 @@
         <v>178</v>
       </c>
       <c r="C30" s="90">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="D30" s="90">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="E30" s="90">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="F30" s="90">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="G30" s="90">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="H30" s="90">
@@ -32973,19 +33005,19 @@
         <v>0.56000000000000005</v>
       </c>
       <c r="L30" s="90">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="M30" s="90">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="N30" s="90">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="O30" s="90">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
     </row>
@@ -32994,39 +33026,39 @@
         <v>179</v>
       </c>
       <c r="C31" s="90">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="D31" s="90">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="E31" s="90">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="F31" s="90">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="G31" s="90">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="H31" s="90">
-        <f t="shared" ref="H31:K34" si="3">IF(H8=1,1,H8*0.9)</f>
+        <f t="shared" ref="H31:K34" si="4">IF(H8=1,1,H8*0.9)</f>
         <v>1</v>
       </c>
       <c r="I31" s="90">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="J31" s="90">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="K31" s="90">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="L31" s="90">
@@ -33047,39 +33079,39 @@
         <v>180</v>
       </c>
       <c r="C32" s="90">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="D32" s="90">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="E32" s="90">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="F32" s="90">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="G32" s="90">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="H32" s="90">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="I32" s="90">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="J32" s="90">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="K32" s="90">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="L32" s="90">
@@ -33100,39 +33132,39 @@
         <v>181</v>
       </c>
       <c r="C33" s="90">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="D33" s="90">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="E33" s="90">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="F33" s="90">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="G33" s="90">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="H33" s="90">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="I33" s="90">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="J33" s="90">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="K33" s="90">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="L33" s="90">
@@ -33170,19 +33202,19 @@
         <v>1</v>
       </c>
       <c r="H34" s="90">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="I34" s="90">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="J34" s="90">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="K34" s="90">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="L34" s="90">
@@ -33251,11 +33283,11 @@
         <v>188</v>
       </c>
       <c r="C36" s="90">
-        <f t="shared" ref="C36:D38" si="4">IF(C13=1,1,C13*0.9)</f>
+        <f t="shared" ref="C36:D38" si="5">IF(C13=1,1,C13*0.9)</f>
         <v>1</v>
       </c>
       <c r="D36" s="90">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="E36" s="90">
@@ -33268,35 +33300,35 @@
         <v>0.62</v>
       </c>
       <c r="H36" s="90">
-        <f t="shared" ref="H36:O36" si="5">IF(H13=1,1,H13*0.9)</f>
+        <f t="shared" ref="H36:O36" si="6">IF(H13=1,1,H13*0.9)</f>
         <v>1</v>
       </c>
       <c r="I36" s="90">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="J36" s="90">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="K36" s="90">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="L36" s="90">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="M36" s="90">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="N36" s="90">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="O36" s="90">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
     </row>
@@ -33305,39 +33337,39 @@
         <v>189</v>
       </c>
       <c r="C37" s="90">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="D37" s="90">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="E37" s="90">
-        <f t="shared" ref="E37:K37" si="6">IF(E14=1,1,E14*0.9)</f>
+        <f t="shared" ref="E37:K37" si="7">IF(E14=1,1,E14*0.9)</f>
         <v>1</v>
       </c>
       <c r="F37" s="90">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="G37" s="90">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="H37" s="90">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="I37" s="90">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="J37" s="90">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="K37" s="90">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="L37" s="90">
@@ -33358,11 +33390,11 @@
         <v>192</v>
       </c>
       <c r="C38" s="90">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="D38" s="90">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="E38" s="90">
@@ -33372,39 +33404,39 @@
         <v>0.3</v>
       </c>
       <c r="G38" s="90">
-        <f t="shared" ref="G38:O38" si="7">IF(G15=1,1,G15*0.9)</f>
+        <f t="shared" ref="G38:O38" si="8">IF(G15=1,1,G15*0.9)</f>
         <v>1</v>
       </c>
       <c r="H38" s="90">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="I38" s="90">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="J38" s="90">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="K38" s="90">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="L38" s="90">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="M38" s="90">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="N38" s="90">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="O38" s="90">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
     </row>
@@ -33419,55 +33451,55 @@
         <v>172</v>
       </c>
       <c r="C41" s="90">
-        <f t="shared" ref="C41:O41" si="8">IF(C18=1,1,C18*0.9)</f>
+        <f t="shared" ref="C41:O41" si="9">IF(C18=1,1,C18*0.9)</f>
         <v>1</v>
       </c>
       <c r="D41" s="90">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>1</v>
       </c>
       <c r="E41" s="90">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>1</v>
       </c>
       <c r="F41" s="90">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>1</v>
       </c>
       <c r="G41" s="90">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>1</v>
       </c>
       <c r="H41" s="90">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>1</v>
       </c>
       <c r="I41" s="90">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>1</v>
       </c>
       <c r="J41" s="90">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>1</v>
       </c>
       <c r="K41" s="90">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>1</v>
       </c>
       <c r="L41" s="90">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>1</v>
       </c>
       <c r="M41" s="90">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>1</v>
       </c>
       <c r="N41" s="90">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>1</v>
       </c>
       <c r="O41" s="90">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>1</v>
       </c>
     </row>
@@ -33476,11 +33508,11 @@
         <v>173</v>
       </c>
       <c r="C42" s="90">
-        <f t="shared" ref="C42:D44" si="9">IF(C19=1,1,C19*0.9)</f>
+        <f t="shared" ref="C42:D44" si="10">IF(C19=1,1,C19*0.9)</f>
         <v>1</v>
       </c>
       <c r="D42" s="90">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>1</v>
       </c>
       <c r="E42" s="90">
@@ -33522,56 +33554,56 @@
         <v>174</v>
       </c>
       <c r="C43" s="90">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>1</v>
       </c>
       <c r="D43" s="90">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>1</v>
       </c>
       <c r="E43" s="90">
-        <f t="shared" ref="E43:O43" si="10">IF(E20=1,1,E20*0.9)</f>
-        <v>1</v>
+        <f t="shared" ref="E43:O43" si="11">IF(E20=1,1,E20*0.9)</f>
+        <v>0.87839999999999996</v>
       </c>
       <c r="F43" s="90">
-        <f t="shared" si="10"/>
-        <v>1</v>
+        <f t="shared" si="11"/>
+        <v>0.87839999999999996</v>
       </c>
       <c r="G43" s="90">
-        <f t="shared" si="10"/>
-        <v>1</v>
+        <f t="shared" si="11"/>
+        <v>0.87839999999999996</v>
       </c>
       <c r="H43" s="90">
-        <f t="shared" si="10"/>
-        <v>1</v>
+        <f t="shared" si="11"/>
+        <v>0.87839999999999996</v>
       </c>
       <c r="I43" s="90">
-        <f t="shared" si="10"/>
-        <v>1</v>
+        <f t="shared" si="11"/>
+        <v>0.87839999999999996</v>
       </c>
       <c r="J43" s="90">
-        <f t="shared" si="10"/>
-        <v>1</v>
+        <f t="shared" si="11"/>
+        <v>0.87839999999999996</v>
       </c>
       <c r="K43" s="90">
-        <f t="shared" si="10"/>
-        <v>1</v>
+        <f t="shared" si="11"/>
+        <v>0.87839999999999996</v>
       </c>
       <c r="L43" s="90">
-        <f t="shared" si="10"/>
-        <v>1</v>
+        <f t="shared" si="11"/>
+        <v>0.87839999999999996</v>
       </c>
       <c r="M43" s="90">
-        <f t="shared" si="10"/>
-        <v>1</v>
+        <f t="shared" si="11"/>
+        <v>0.87839999999999996</v>
       </c>
       <c r="N43" s="90">
-        <f t="shared" si="10"/>
-        <v>1</v>
+        <f t="shared" si="11"/>
+        <v>0.87839999999999996</v>
       </c>
       <c r="O43" s="90">
-        <f t="shared" si="10"/>
-        <v>1</v>
+        <f t="shared" si="11"/>
+        <v>0.87839999999999996</v>
       </c>
     </row>
     <row r="44" spans="1:15" x14ac:dyDescent="0.25">
@@ -33579,11 +33611,11 @@
         <v>182</v>
       </c>
       <c r="C44" s="90">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>1</v>
       </c>
       <c r="D44" s="90">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>1</v>
       </c>
       <c r="E44" s="90">
@@ -33684,47 +33716,47 @@
         <v>0.7</v>
       </c>
       <c r="E49" s="90">
-        <f t="shared" ref="E49:O49" si="11">IF(E3=1,1,E3*1.05)</f>
+        <f t="shared" ref="E49:O49" si="12">IF(E3=1,1,E3*1.05)</f>
         <v>1</v>
       </c>
       <c r="F49" s="90">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>1</v>
       </c>
       <c r="G49" s="90">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>1</v>
       </c>
       <c r="H49" s="90">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>1</v>
       </c>
       <c r="I49" s="90">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>1</v>
       </c>
       <c r="J49" s="90">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>1</v>
       </c>
       <c r="K49" s="90">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>1</v>
       </c>
       <c r="L49" s="90">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>1</v>
       </c>
       <c r="M49" s="90">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>1</v>
       </c>
       <c r="N49" s="90">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>1</v>
       </c>
       <c r="O49" s="90">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>1</v>
       </c>
     </row>
@@ -33733,23 +33765,23 @@
         <v>175</v>
       </c>
       <c r="C50" s="90">
-        <f t="shared" ref="C50:G56" si="12">IF(C4=1,1,C4*1.05)</f>
+        <f t="shared" ref="C50:G56" si="13">IF(C4=1,1,C4*1.05)</f>
         <v>1</v>
       </c>
       <c r="D50" s="90">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="E50" s="90">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="F50" s="90">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="G50" s="90">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="H50" s="90">
@@ -33765,19 +33797,19 @@
         <v>0.95</v>
       </c>
       <c r="L50" s="90">
-        <f t="shared" ref="L50:O53" si="13">IF(L4=1,1,L4*1.05)</f>
+        <f t="shared" ref="L50:O53" si="14">IF(L4=1,1,L4*1.05)</f>
         <v>1</v>
       </c>
       <c r="M50" s="90">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>1</v>
       </c>
       <c r="N50" s="90">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>1</v>
       </c>
       <c r="O50" s="90">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>1</v>
       </c>
     </row>
@@ -33786,23 +33818,23 @@
         <v>176</v>
       </c>
       <c r="C51" s="90">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="D51" s="90">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="E51" s="90">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="F51" s="90">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="G51" s="90">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="H51" s="90">
@@ -33818,19 +33850,19 @@
         <v>0.95</v>
       </c>
       <c r="L51" s="90">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>1</v>
       </c>
       <c r="M51" s="90">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>1</v>
       </c>
       <c r="N51" s="90">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>1</v>
       </c>
       <c r="O51" s="90">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>1</v>
       </c>
     </row>
@@ -33839,23 +33871,23 @@
         <v>177</v>
       </c>
       <c r="C52" s="90">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="D52" s="90">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="E52" s="90">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="F52" s="90">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="G52" s="90">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="H52" s="90">
@@ -33871,19 +33903,19 @@
         <v>0.95</v>
       </c>
       <c r="L52" s="90">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>1</v>
       </c>
       <c r="M52" s="90">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>1</v>
       </c>
       <c r="N52" s="90">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>1</v>
       </c>
       <c r="O52" s="90">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>1</v>
       </c>
     </row>
@@ -33892,23 +33924,23 @@
         <v>178</v>
       </c>
       <c r="C53" s="90">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="D53" s="90">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="E53" s="90">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="F53" s="90">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="G53" s="90">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="H53" s="90">
@@ -33924,19 +33956,19 @@
         <v>0.95</v>
       </c>
       <c r="L53" s="90">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>1</v>
       </c>
       <c r="M53" s="90">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>1</v>
       </c>
       <c r="N53" s="90">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>1</v>
       </c>
       <c r="O53" s="90">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>1</v>
       </c>
     </row>
@@ -33945,39 +33977,39 @@
         <v>179</v>
       </c>
       <c r="C54" s="90">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="D54" s="90">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="E54" s="90">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="F54" s="90">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="G54" s="90">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="H54" s="90">
-        <f t="shared" ref="H54:K57" si="14">IF(H8=1,1,H8*1.05)</f>
+        <f t="shared" ref="H54:K57" si="15">IF(H8=1,1,H8*1.05)</f>
         <v>1</v>
       </c>
       <c r="I54" s="90">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="J54" s="90">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="K54" s="90">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="L54" s="90">
@@ -33998,39 +34030,39 @@
         <v>180</v>
       </c>
       <c r="C55" s="90">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="D55" s="90">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="E55" s="90">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="F55" s="90">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="G55" s="90">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="H55" s="90">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="I55" s="90">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="J55" s="90">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="K55" s="90">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="L55" s="90">
@@ -34051,39 +34083,39 @@
         <v>181</v>
       </c>
       <c r="C56" s="90">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="D56" s="90">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="E56" s="90">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="F56" s="90">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="G56" s="90">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="H56" s="90">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="I56" s="90">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="J56" s="90">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="K56" s="90">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="L56" s="90">
@@ -34122,19 +34154,19 @@
         <v>1</v>
       </c>
       <c r="H57" s="90">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="I57" s="90">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="J57" s="90">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="K57" s="90">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>1</v>
       </c>
       <c r="L57" s="90">
@@ -34203,11 +34235,11 @@
         <v>188</v>
       </c>
       <c r="C59" s="90">
-        <f t="shared" ref="C59:D61" si="15">IF(C13=1,1,C13*1.05)</f>
+        <f t="shared" ref="C59:D61" si="16">IF(C13=1,1,C13*1.05)</f>
         <v>1</v>
       </c>
       <c r="D59" s="90">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>1</v>
       </c>
       <c r="E59" s="90">
@@ -34220,35 +34252,35 @@
         <v>0.77</v>
       </c>
       <c r="H59" s="90">
-        <f t="shared" ref="H59:O59" si="16">IF(H13=1,1,H13*1.05)</f>
+        <f t="shared" ref="H59:O59" si="17">IF(H13=1,1,H13*1.05)</f>
         <v>1</v>
       </c>
       <c r="I59" s="90">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>1</v>
       </c>
       <c r="J59" s="90">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>1</v>
       </c>
       <c r="K59" s="90">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>1</v>
       </c>
       <c r="L59" s="90">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>1</v>
       </c>
       <c r="M59" s="90">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>1</v>
       </c>
       <c r="N59" s="90">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>1</v>
       </c>
       <c r="O59" s="90">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>1</v>
       </c>
     </row>
@@ -34257,39 +34289,39 @@
         <v>189</v>
       </c>
       <c r="C60" s="90">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>1</v>
       </c>
       <c r="D60" s="90">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>1</v>
       </c>
       <c r="E60" s="90">
-        <f t="shared" ref="E60:K60" si="17">IF(E14=1,1,E14*1.05)</f>
+        <f t="shared" ref="E60:K60" si="18">IF(E14=1,1,E14*1.05)</f>
         <v>1</v>
       </c>
       <c r="F60" s="90">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>1</v>
       </c>
       <c r="G60" s="90">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>1</v>
       </c>
       <c r="H60" s="90">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>1</v>
       </c>
       <c r="I60" s="90">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>1</v>
       </c>
       <c r="J60" s="90">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>1</v>
       </c>
       <c r="K60" s="90">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>1</v>
       </c>
       <c r="L60" s="90">
@@ -34310,11 +34342,11 @@
         <v>192</v>
       </c>
       <c r="C61" s="90">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>1</v>
       </c>
       <c r="D61" s="90">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>1</v>
       </c>
       <c r="E61" s="90">
@@ -34324,39 +34356,39 @@
         <v>0.44</v>
       </c>
       <c r="G61" s="90">
-        <f t="shared" ref="G61:O61" si="18">IF(G15=1,1,G15*1.05)</f>
+        <f t="shared" ref="G61:O61" si="19">IF(G15=1,1,G15*1.05)</f>
         <v>1</v>
       </c>
       <c r="H61" s="90">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>1</v>
       </c>
       <c r="I61" s="90">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>1</v>
       </c>
       <c r="J61" s="90">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>1</v>
       </c>
       <c r="K61" s="90">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>1</v>
       </c>
       <c r="L61" s="90">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>1</v>
       </c>
       <c r="M61" s="90">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>1</v>
       </c>
       <c r="N61" s="90">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>1</v>
       </c>
       <c r="O61" s="90">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>1</v>
       </c>
     </row>
@@ -34371,55 +34403,55 @@
         <v>172</v>
       </c>
       <c r="C64" s="90">
-        <f t="shared" ref="C64:O64" si="19">IF(C18=1,1,C18*1.05)</f>
+        <f t="shared" ref="C64:O64" si="20">IF(C18=1,1,C18*1.05)</f>
         <v>1</v>
       </c>
       <c r="D64" s="90">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>1</v>
       </c>
       <c r="E64" s="90">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>1</v>
       </c>
       <c r="F64" s="90">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>1</v>
       </c>
       <c r="G64" s="90">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>1</v>
       </c>
       <c r="H64" s="90">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>1</v>
       </c>
       <c r="I64" s="90">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>1</v>
       </c>
       <c r="J64" s="90">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>1</v>
       </c>
       <c r="K64" s="90">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>1</v>
       </c>
       <c r="L64" s="90">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>1</v>
       </c>
       <c r="M64" s="90">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>1</v>
       </c>
       <c r="N64" s="90">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>1</v>
       </c>
       <c r="O64" s="90">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>1</v>
       </c>
     </row>
@@ -34428,11 +34460,11 @@
         <v>173</v>
       </c>
       <c r="C65" s="90">
-        <f t="shared" ref="C65:D67" si="20">IF(C19=1,1,C19*1.05)</f>
+        <f t="shared" ref="C65:D67" si="21">IF(C19=1,1,C19*1.05)</f>
         <v>1</v>
       </c>
       <c r="D65" s="90">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>1</v>
       </c>
       <c r="E65" s="90">
@@ -34474,56 +34506,56 @@
         <v>174</v>
       </c>
       <c r="C66" s="90">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>1</v>
       </c>
       <c r="D66" s="90">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>1</v>
       </c>
       <c r="E66" s="90">
-        <f t="shared" ref="E66:O66" si="21">IF(E20=1,1,E20*1.05)</f>
-        <v>1</v>
+        <f t="shared" ref="E66:O66" si="22">IF(E20=1,1,E20*1.05)</f>
+        <v>1.0247999999999999</v>
       </c>
       <c r="F66" s="90">
-        <f t="shared" si="21"/>
-        <v>1</v>
+        <f t="shared" si="22"/>
+        <v>1.0247999999999999</v>
       </c>
       <c r="G66" s="90">
-        <f t="shared" si="21"/>
-        <v>1</v>
+        <f t="shared" si="22"/>
+        <v>1.0247999999999999</v>
       </c>
       <c r="H66" s="90">
-        <f t="shared" si="21"/>
-        <v>1</v>
+        <f t="shared" si="22"/>
+        <v>1.0247999999999999</v>
       </c>
       <c r="I66" s="90">
-        <f t="shared" si="21"/>
-        <v>1</v>
+        <f t="shared" si="22"/>
+        <v>1.0247999999999999</v>
       </c>
       <c r="J66" s="90">
-        <f t="shared" si="21"/>
-        <v>1</v>
+        <f t="shared" si="22"/>
+        <v>1.0247999999999999</v>
       </c>
       <c r="K66" s="90">
-        <f t="shared" si="21"/>
-        <v>1</v>
+        <f t="shared" si="22"/>
+        <v>1.0247999999999999</v>
       </c>
       <c r="L66" s="90">
-        <f t="shared" si="21"/>
-        <v>1</v>
+        <f t="shared" si="22"/>
+        <v>1.0247999999999999</v>
       </c>
       <c r="M66" s="90">
-        <f t="shared" si="21"/>
-        <v>1</v>
+        <f t="shared" si="22"/>
+        <v>1.0247999999999999</v>
       </c>
       <c r="N66" s="90">
-        <f t="shared" si="21"/>
-        <v>1</v>
+        <f t="shared" si="22"/>
+        <v>1.0247999999999999</v>
       </c>
       <c r="O66" s="90">
-        <f t="shared" si="21"/>
-        <v>1</v>
+        <f t="shared" si="22"/>
+        <v>1.0247999999999999</v>
       </c>
     </row>
     <row r="67" spans="2:15" x14ac:dyDescent="0.25">
@@ -34531,11 +34563,11 @@
         <v>182</v>
       </c>
       <c r="C67" s="90">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>1</v>
       </c>
       <c r="D67" s="90">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>1</v>
       </c>
       <c r="E67" s="90">
@@ -40665,177 +40697,4 @@
   <sheetProtection algorithmName="SHA-512" hashValue="tS5A5il384gB8zsJjwidwZIpdVsJo/ah59cRAmnHpig36ZssdSIeiIXxiNqdW+7yhHG743nXUgYflxFLjdX6Kg==" saltValue="H9BMcvjdiLgSEjFGZvTrQw==" spinCount="100000" sheet="1" scenarios="1" selectLockedCells="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100856A3DB4B0A5FF4A85E5854FA9B1BD84" ma:contentTypeVersion="6" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="107b52809c0cc4b5077f1ac81d3c69cc">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5de2aea6-bdc3-4e5f-b0ae-84d85b5764e4" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="82b7e1b740270cfb0676be859a78f3d0" ns2:_="">
-    <xsd:import namespace="5de2aea6-bdc3-4e5f-b0ae-84d85b5764e4"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="5de2aea6-bdc3-4e5f-b0ae-84d85b5764e4" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="10" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="11" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="12" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BD5E8882-0615-453B-8A7B-3E777EC54E25}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6640C4EA-3EE7-491A-98B6-71B785ABC1DC}"/>
 </file>
</xml_diff>